<commit_message>
Export formatted Excel pink sheet
</commit_message>
<xml_diff>
--- a/data/pink_sheet.xlsx
+++ b/data/pink_sheet.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -27,6 +27,11 @@
     </font>
     <font>
       <name val="Arial"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -50,10 +55,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -890,7 +898,7 @@
     <col width="10" customWidth="1" min="465" max="465"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="60" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Date</t>
@@ -3218,946 +3226,946 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>2026-04-26</t>
         </is>
       </c>
-      <c r="B2" s="1" t="inlineStr"/>
-      <c r="C2" s="1" t="inlineStr"/>
-      <c r="D2" s="1" t="inlineStr"/>
-      <c r="E2" s="1" t="inlineStr"/>
-      <c r="F2" s="1" t="inlineStr"/>
-      <c r="G2" s="1" t="inlineStr"/>
-      <c r="H2" s="1" t="inlineStr"/>
-      <c r="I2" s="1" t="inlineStr"/>
-      <c r="J2" s="1" t="inlineStr"/>
-      <c r="K2" s="1" t="inlineStr"/>
-      <c r="L2" s="1" t="inlineStr"/>
-      <c r="M2" s="1" t="inlineStr"/>
-      <c r="N2" s="1" t="inlineStr"/>
-      <c r="O2" s="1" t="inlineStr"/>
-      <c r="P2" s="1" t="inlineStr"/>
-      <c r="Q2" s="1" t="inlineStr"/>
-      <c r="R2" s="1" t="inlineStr"/>
-      <c r="S2" s="1" t="inlineStr"/>
-      <c r="T2" s="1" t="inlineStr"/>
-      <c r="U2" s="1" t="inlineStr"/>
-      <c r="V2" s="1" t="inlineStr"/>
-      <c r="W2" s="1" t="inlineStr"/>
-      <c r="X2" s="1" t="inlineStr"/>
-      <c r="Y2" s="1" t="inlineStr"/>
-      <c r="Z2" s="1" t="inlineStr"/>
-      <c r="AA2" s="1" t="inlineStr"/>
-      <c r="AB2" s="1" t="inlineStr"/>
-      <c r="AC2" s="1" t="inlineStr"/>
-      <c r="AD2" s="1" t="inlineStr"/>
-      <c r="AE2" s="1" t="inlineStr"/>
-      <c r="AF2" s="1" t="inlineStr"/>
-      <c r="AG2" s="1" t="inlineStr"/>
-      <c r="AH2" s="1" t="inlineStr"/>
-      <c r="AI2" s="1" t="inlineStr"/>
-      <c r="AJ2" s="1" t="inlineStr"/>
-      <c r="AK2" s="1" t="inlineStr"/>
-      <c r="AL2" s="1" t="inlineStr"/>
-      <c r="AM2" s="1" t="inlineStr"/>
-      <c r="AN2" s="1" t="inlineStr"/>
-      <c r="AO2" s="1" t="inlineStr"/>
-      <c r="AP2" s="1" t="inlineStr"/>
-      <c r="AQ2" s="1" t="inlineStr"/>
-      <c r="AR2" s="1" t="inlineStr"/>
-      <c r="AS2" s="1" t="inlineStr"/>
-      <c r="AT2" s="1" t="inlineStr"/>
-      <c r="AU2" s="1" t="inlineStr"/>
-      <c r="AV2" s="1" t="inlineStr"/>
-      <c r="AW2" s="1" t="inlineStr"/>
-      <c r="AX2" s="1" t="inlineStr"/>
-      <c r="AY2" s="1" t="inlineStr"/>
-      <c r="AZ2" s="1" t="inlineStr"/>
-      <c r="BA2" s="1" t="inlineStr"/>
-      <c r="BB2" s="1" t="inlineStr"/>
-      <c r="BC2" s="1" t="inlineStr"/>
-      <c r="BD2" s="1" t="inlineStr"/>
-      <c r="BE2" s="1" t="inlineStr"/>
-      <c r="BF2" s="1" t="inlineStr"/>
-      <c r="BG2" s="1" t="inlineStr"/>
-      <c r="BH2" s="1" t="inlineStr"/>
-      <c r="BI2" s="1" t="inlineStr"/>
-      <c r="BJ2" s="1" t="inlineStr"/>
-      <c r="BK2" s="1" t="inlineStr"/>
-      <c r="BL2" s="1" t="inlineStr"/>
-      <c r="BM2" s="1" t="inlineStr"/>
-      <c r="BN2" s="1" t="inlineStr"/>
-      <c r="BO2" s="1" t="inlineStr"/>
-      <c r="BP2" s="1" t="inlineStr"/>
-      <c r="BQ2" s="1" t="inlineStr"/>
-      <c r="BR2" s="1" t="inlineStr"/>
-      <c r="BS2" s="1" t="inlineStr"/>
-      <c r="BT2" s="1" t="inlineStr"/>
-      <c r="BU2" s="1" t="inlineStr"/>
-      <c r="BV2" s="1" t="inlineStr"/>
-      <c r="BW2" s="1" t="inlineStr"/>
-      <c r="BX2" s="1" t="inlineStr"/>
-      <c r="BY2" s="1" t="inlineStr"/>
-      <c r="BZ2" s="1" t="inlineStr"/>
-      <c r="CA2" s="1" t="inlineStr"/>
-      <c r="CB2" s="1" t="inlineStr"/>
-      <c r="CC2" s="1" t="inlineStr"/>
-      <c r="CD2" s="1" t="inlineStr"/>
-      <c r="CE2" s="1" t="inlineStr"/>
-      <c r="CF2" s="1" t="inlineStr"/>
-      <c r="CG2" s="1" t="inlineStr"/>
-      <c r="CH2" s="1" t="inlineStr"/>
-      <c r="CI2" s="1" t="inlineStr"/>
-      <c r="CJ2" s="1" t="inlineStr"/>
-      <c r="CK2" s="1" t="inlineStr"/>
-      <c r="CL2" s="1" t="inlineStr"/>
-      <c r="CM2" s="1" t="inlineStr"/>
-      <c r="CN2" s="1" t="inlineStr"/>
-      <c r="CO2" s="1" t="inlineStr"/>
-      <c r="CP2" s="1" t="inlineStr"/>
-      <c r="CQ2" s="1" t="inlineStr"/>
-      <c r="CR2" s="1" t="inlineStr"/>
-      <c r="CS2" s="1" t="inlineStr"/>
-      <c r="CT2" s="1" t="inlineStr"/>
-      <c r="CU2" s="1" t="inlineStr"/>
-      <c r="CV2" s="1" t="inlineStr"/>
-      <c r="CW2" s="1" t="inlineStr"/>
-      <c r="CX2" s="1" t="inlineStr"/>
-      <c r="CY2" s="1" t="inlineStr"/>
-      <c r="CZ2" s="1" t="inlineStr"/>
-      <c r="DA2" s="1" t="inlineStr"/>
-      <c r="DB2" s="1" t="inlineStr"/>
-      <c r="DC2" s="1" t="inlineStr"/>
-      <c r="DD2" s="1" t="inlineStr"/>
-      <c r="DE2" s="1" t="inlineStr"/>
-      <c r="DF2" s="1" t="inlineStr"/>
-      <c r="DG2" s="1" t="inlineStr"/>
-      <c r="DH2" s="1" t="inlineStr"/>
-      <c r="DI2" s="1" t="inlineStr"/>
-      <c r="DJ2" s="1" t="inlineStr"/>
-      <c r="DK2" s="1" t="inlineStr"/>
-      <c r="DL2" s="1" t="inlineStr"/>
-      <c r="DM2" s="1" t="inlineStr"/>
-      <c r="DN2" s="1" t="inlineStr"/>
-      <c r="DO2" s="1" t="inlineStr"/>
-      <c r="DP2" s="1" t="inlineStr"/>
-      <c r="DQ2" s="1" t="inlineStr"/>
-      <c r="DR2" s="1" t="inlineStr"/>
-      <c r="DS2" s="1" t="inlineStr"/>
-      <c r="DT2" s="1" t="inlineStr"/>
-      <c r="DU2" s="1" t="inlineStr"/>
-      <c r="DV2" s="1" t="inlineStr"/>
-      <c r="DW2" s="1" t="inlineStr"/>
-      <c r="DX2" s="1" t="inlineStr"/>
-      <c r="DY2" s="1" t="inlineStr"/>
-      <c r="DZ2" s="1" t="inlineStr"/>
-      <c r="EA2" s="1" t="inlineStr"/>
-      <c r="EB2" s="1" t="inlineStr"/>
-      <c r="EC2" s="1" t="inlineStr"/>
-      <c r="ED2" s="1" t="inlineStr"/>
-      <c r="EE2" s="1" t="inlineStr"/>
-      <c r="EF2" s="1" t="inlineStr"/>
-      <c r="EG2" s="1" t="inlineStr"/>
-      <c r="EH2" s="1" t="inlineStr"/>
-      <c r="EI2" s="1" t="inlineStr"/>
-      <c r="EJ2" s="1" t="inlineStr"/>
-      <c r="EK2" s="1" t="inlineStr"/>
-      <c r="EL2" s="1" t="inlineStr"/>
-      <c r="EM2" s="1" t="inlineStr"/>
-      <c r="EN2" s="1" t="inlineStr"/>
-      <c r="EO2" s="1" t="inlineStr"/>
-      <c r="EP2" s="1" t="inlineStr"/>
-      <c r="EQ2" s="1" t="inlineStr"/>
-      <c r="ER2" s="1" t="inlineStr"/>
-      <c r="ES2" s="1" t="inlineStr"/>
-      <c r="ET2" s="1" t="inlineStr"/>
-      <c r="EU2" s="1" t="inlineStr"/>
-      <c r="EV2" s="1" t="inlineStr"/>
-      <c r="EW2" s="1" t="inlineStr"/>
-      <c r="EX2" s="1" t="inlineStr"/>
-      <c r="EY2" s="1" t="inlineStr"/>
-      <c r="EZ2" s="1" t="inlineStr"/>
-      <c r="FA2" s="1" t="inlineStr"/>
-      <c r="FB2" s="1" t="inlineStr"/>
-      <c r="FC2" s="1" t="inlineStr"/>
-      <c r="FD2" s="1" t="inlineStr"/>
-      <c r="FE2" s="1" t="inlineStr"/>
-      <c r="FF2" s="1" t="inlineStr"/>
-      <c r="FG2" s="1" t="inlineStr"/>
-      <c r="FH2" s="1" t="inlineStr"/>
-      <c r="FI2" s="1" t="inlineStr"/>
-      <c r="FJ2" s="1" t="inlineStr"/>
-      <c r="FK2" s="1" t="inlineStr"/>
-      <c r="FL2" s="1" t="inlineStr"/>
-      <c r="FM2" s="1" t="inlineStr"/>
-      <c r="FN2" s="1" t="inlineStr"/>
-      <c r="FO2" s="1" t="inlineStr"/>
-      <c r="FP2" s="1" t="inlineStr"/>
-      <c r="FQ2" s="1" t="inlineStr"/>
-      <c r="FR2" s="1" t="inlineStr"/>
-      <c r="FS2" s="1" t="inlineStr"/>
-      <c r="FT2" s="1" t="inlineStr"/>
-      <c r="FU2" s="1" t="inlineStr"/>
-      <c r="FV2" s="1" t="inlineStr"/>
-      <c r="FW2" s="1" t="inlineStr"/>
-      <c r="FX2" s="1" t="inlineStr"/>
-      <c r="FY2" s="1" t="inlineStr"/>
-      <c r="FZ2" s="1" t="inlineStr"/>
-      <c r="GA2" s="1" t="inlineStr"/>
-      <c r="GB2" s="1" t="inlineStr"/>
-      <c r="GC2" s="1" t="inlineStr"/>
-      <c r="GD2" s="1" t="inlineStr"/>
-      <c r="GE2" s="1" t="inlineStr"/>
-      <c r="GF2" s="1" t="inlineStr"/>
-      <c r="GG2" s="1" t="inlineStr"/>
-      <c r="GH2" s="1" t="inlineStr"/>
-      <c r="GI2" s="1" t="inlineStr"/>
-      <c r="GJ2" s="1" t="inlineStr"/>
-      <c r="GK2" s="1" t="inlineStr"/>
-      <c r="GL2" s="1" t="inlineStr"/>
-      <c r="GM2" s="1" t="inlineStr"/>
-      <c r="GN2" s="1" t="inlineStr"/>
-      <c r="GO2" s="1" t="inlineStr"/>
-      <c r="GP2" s="1" t="inlineStr"/>
-      <c r="GQ2" s="1" t="inlineStr"/>
-      <c r="GR2" s="1" t="inlineStr"/>
-      <c r="GS2" s="1" t="inlineStr"/>
-      <c r="GT2" s="1" t="inlineStr"/>
-      <c r="GU2" s="1" t="inlineStr"/>
-      <c r="GV2" s="1" t="inlineStr"/>
-      <c r="GW2" s="1" t="inlineStr"/>
-      <c r="GX2" s="1" t="inlineStr"/>
-      <c r="GY2" s="1" t="inlineStr"/>
-      <c r="GZ2" s="1" t="inlineStr"/>
-      <c r="HA2" s="1" t="inlineStr"/>
-      <c r="HB2" s="1" t="inlineStr"/>
-      <c r="HC2" s="1" t="inlineStr"/>
-      <c r="HD2" s="1" t="inlineStr"/>
-      <c r="HE2" s="1" t="inlineStr"/>
-      <c r="HF2" s="1" t="inlineStr"/>
-      <c r="HG2" s="1" t="inlineStr"/>
-      <c r="HH2" s="1" t="inlineStr"/>
-      <c r="HI2" s="1" t="inlineStr"/>
-      <c r="HJ2" s="1" t="inlineStr"/>
-      <c r="HK2" s="1" t="inlineStr"/>
-      <c r="HL2" s="1" t="inlineStr"/>
-      <c r="HM2" s="1" t="inlineStr"/>
-      <c r="HN2" s="1" t="inlineStr"/>
-      <c r="HO2" s="1" t="inlineStr"/>
-      <c r="HP2" s="1" t="inlineStr"/>
-      <c r="HQ2" s="1" t="inlineStr"/>
-      <c r="HR2" s="1" t="inlineStr"/>
-      <c r="HS2" s="1" t="inlineStr"/>
-      <c r="HT2" s="1" t="inlineStr"/>
-      <c r="HU2" s="1" t="inlineStr"/>
-      <c r="HV2" s="1" t="inlineStr"/>
-      <c r="HW2" s="1" t="inlineStr"/>
-      <c r="HX2" s="1" t="inlineStr"/>
-      <c r="HY2" s="1" t="inlineStr"/>
-      <c r="HZ2" s="1" t="inlineStr"/>
-      <c r="IA2" s="1" t="inlineStr"/>
-      <c r="IB2" s="1" t="inlineStr"/>
-      <c r="IC2" s="1" t="inlineStr"/>
-      <c r="ID2" s="1" t="inlineStr"/>
-      <c r="IE2" s="1" t="inlineStr"/>
-      <c r="IF2" s="1" t="inlineStr"/>
-      <c r="IG2" s="1" t="inlineStr"/>
-      <c r="IH2" s="1" t="inlineStr"/>
-      <c r="II2" s="1" t="inlineStr"/>
-      <c r="IJ2" s="1" t="inlineStr"/>
-      <c r="IK2" s="1" t="inlineStr"/>
-      <c r="IL2" s="1" t="inlineStr"/>
-      <c r="IM2" s="1" t="inlineStr"/>
-      <c r="IN2" s="1" t="inlineStr"/>
-      <c r="IO2" s="1" t="inlineStr"/>
-      <c r="IP2" s="1" t="inlineStr"/>
-      <c r="IQ2" s="1" t="inlineStr"/>
-      <c r="IR2" s="1" t="inlineStr"/>
-      <c r="IS2" s="1" t="inlineStr"/>
-      <c r="IT2" s="1" t="inlineStr"/>
-      <c r="IU2" s="1" t="inlineStr"/>
-      <c r="IV2" s="1" t="inlineStr"/>
-      <c r="IW2" s="1" t="inlineStr"/>
-      <c r="IX2" s="1" t="inlineStr"/>
-      <c r="IY2" s="1" t="inlineStr"/>
-      <c r="IZ2" s="1" t="inlineStr"/>
-      <c r="JA2" s="1" t="inlineStr"/>
-      <c r="JB2" s="1" t="inlineStr"/>
-      <c r="JC2" s="1" t="inlineStr"/>
-      <c r="JD2" s="1" t="inlineStr"/>
-      <c r="JE2" s="1" t="inlineStr"/>
-      <c r="JF2" s="1" t="inlineStr"/>
-      <c r="JG2" s="1" t="inlineStr"/>
-      <c r="JH2" s="1" t="inlineStr"/>
-      <c r="JI2" s="1" t="inlineStr"/>
-      <c r="JJ2" s="1" t="inlineStr"/>
-      <c r="JK2" s="1" t="inlineStr"/>
-      <c r="JL2" s="1" t="inlineStr"/>
-      <c r="JM2" s="1" t="inlineStr"/>
-      <c r="JN2" s="1" t="inlineStr"/>
-      <c r="JO2" s="1" t="inlineStr"/>
-      <c r="JP2" s="1" t="inlineStr"/>
-      <c r="JQ2" s="1" t="inlineStr"/>
-      <c r="JR2" s="1" t="inlineStr"/>
-      <c r="JS2" s="1" t="inlineStr"/>
-      <c r="JT2" s="1" t="inlineStr"/>
-      <c r="JU2" s="1" t="inlineStr"/>
-      <c r="JV2" s="1" t="inlineStr"/>
-      <c r="JW2" s="1" t="inlineStr"/>
-      <c r="JX2" s="1" t="inlineStr"/>
-      <c r="JY2" s="1" t="inlineStr"/>
-      <c r="JZ2" s="1" t="inlineStr"/>
-      <c r="KA2" s="1" t="inlineStr"/>
-      <c r="KB2" s="1" t="inlineStr"/>
-      <c r="KC2" s="1" t="inlineStr"/>
-      <c r="KD2" s="1" t="inlineStr"/>
-      <c r="KE2" s="1" t="inlineStr"/>
-      <c r="KF2" s="1" t="inlineStr"/>
-      <c r="KG2" s="1" t="inlineStr"/>
-      <c r="KH2" s="1" t="inlineStr"/>
-      <c r="KI2" s="1" t="inlineStr"/>
-      <c r="KJ2" s="1" t="inlineStr"/>
-      <c r="KK2" s="1" t="inlineStr"/>
-      <c r="KL2" s="1" t="inlineStr"/>
-      <c r="KM2" s="1" t="inlineStr"/>
-      <c r="KN2" s="1" t="inlineStr"/>
-      <c r="KO2" s="1" t="inlineStr"/>
-      <c r="KP2" s="1" t="inlineStr"/>
-      <c r="KQ2" s="1" t="inlineStr"/>
-      <c r="KR2" s="1" t="inlineStr"/>
-      <c r="KS2" s="1" t="inlineStr"/>
-      <c r="KT2" s="1" t="inlineStr"/>
-      <c r="KU2" s="1" t="inlineStr"/>
-      <c r="KV2" s="1" t="inlineStr"/>
-      <c r="KW2" s="1" t="inlineStr"/>
-      <c r="KX2" s="1" t="inlineStr"/>
-      <c r="KY2" s="1" t="inlineStr"/>
-      <c r="KZ2" s="1" t="inlineStr"/>
-      <c r="LA2" s="1" t="inlineStr"/>
-      <c r="LB2" s="1" t="inlineStr"/>
-      <c r="LC2" s="1" t="inlineStr"/>
-      <c r="LD2" s="1" t="inlineStr"/>
-      <c r="LE2" s="1" t="inlineStr"/>
-      <c r="LF2" s="1" t="inlineStr"/>
-      <c r="LG2" s="1" t="inlineStr"/>
-      <c r="LH2" s="1" t="inlineStr"/>
-      <c r="LI2" s="1" t="inlineStr"/>
-      <c r="LJ2" s="1" t="inlineStr"/>
-      <c r="LK2" s="1" t="inlineStr"/>
-      <c r="LL2" s="1" t="inlineStr"/>
-      <c r="LM2" s="1" t="inlineStr"/>
-      <c r="LN2" s="1" t="inlineStr"/>
-      <c r="LO2" s="1" t="inlineStr"/>
-      <c r="LP2" s="1" t="inlineStr"/>
-      <c r="LQ2" s="1" t="inlineStr"/>
-      <c r="LR2" s="1" t="inlineStr"/>
-      <c r="LS2" s="1" t="inlineStr"/>
-      <c r="LT2" s="1" t="inlineStr"/>
-      <c r="LU2" s="1" t="inlineStr"/>
-      <c r="LV2" s="1" t="inlineStr"/>
-      <c r="LW2" s="1" t="inlineStr"/>
-      <c r="LX2" s="1" t="inlineStr"/>
-      <c r="LY2" s="1" t="inlineStr"/>
-      <c r="LZ2" s="1" t="inlineStr"/>
-      <c r="MA2" s="1" t="inlineStr"/>
-      <c r="MB2" s="1" t="inlineStr"/>
-      <c r="MC2" s="1" t="inlineStr"/>
-      <c r="MD2" s="1" t="inlineStr"/>
-      <c r="ME2" s="1" t="inlineStr"/>
-      <c r="MF2" s="1" t="inlineStr"/>
-      <c r="MG2" s="1" t="inlineStr"/>
-      <c r="MH2" s="1" t="inlineStr"/>
-      <c r="MI2" s="1" t="inlineStr"/>
-      <c r="MJ2" s="1" t="inlineStr"/>
-      <c r="MK2" s="1" t="inlineStr"/>
-      <c r="ML2" s="1" t="inlineStr"/>
-      <c r="MM2" s="1" t="inlineStr"/>
-      <c r="MN2" s="1" t="inlineStr"/>
-      <c r="MO2" s="1" t="inlineStr"/>
-      <c r="MP2" s="1" t="inlineStr"/>
-      <c r="MQ2" s="1" t="inlineStr"/>
-      <c r="MR2" s="1" t="inlineStr"/>
-      <c r="MS2" s="1" t="inlineStr"/>
-      <c r="MT2" s="1" t="inlineStr"/>
-      <c r="MU2" s="1" t="inlineStr"/>
-      <c r="MV2" s="1" t="inlineStr"/>
-      <c r="MW2" s="1" t="inlineStr"/>
-      <c r="MX2" s="1" t="inlineStr"/>
-      <c r="MY2" s="1" t="inlineStr"/>
-      <c r="MZ2" s="1" t="inlineStr"/>
-      <c r="NA2" s="1" t="inlineStr"/>
-      <c r="NB2" s="1" t="inlineStr"/>
-      <c r="NC2" s="1" t="inlineStr"/>
-      <c r="ND2" s="1" t="inlineStr"/>
-      <c r="NE2" s="1" t="inlineStr"/>
-      <c r="NF2" s="1" t="inlineStr"/>
-      <c r="NG2" s="1" t="inlineStr"/>
-      <c r="NH2" s="1" t="inlineStr"/>
-      <c r="NI2" s="1" t="inlineStr"/>
-      <c r="NJ2" s="1" t="inlineStr"/>
-      <c r="NK2" s="1" t="inlineStr"/>
-      <c r="NL2" s="1" t="inlineStr"/>
-      <c r="NM2" s="1" t="inlineStr"/>
-      <c r="NN2" s="1" t="inlineStr"/>
-      <c r="NO2" s="1" t="inlineStr"/>
-      <c r="NP2" s="1" t="inlineStr"/>
-      <c r="NQ2" s="1" t="inlineStr"/>
-      <c r="NR2" s="1" t="inlineStr"/>
-      <c r="NS2" s="1" t="inlineStr"/>
-      <c r="NT2" s="1" t="inlineStr"/>
-      <c r="NU2" s="1" t="inlineStr"/>
-      <c r="NV2" s="1" t="inlineStr"/>
-      <c r="NW2" s="1" t="inlineStr"/>
-      <c r="NX2" s="1" t="inlineStr"/>
-      <c r="NY2" s="1" t="inlineStr"/>
-      <c r="NZ2" s="1" t="inlineStr"/>
-      <c r="OA2" s="1" t="inlineStr"/>
-      <c r="OB2" s="1" t="inlineStr"/>
-      <c r="OC2" s="1" t="inlineStr"/>
-      <c r="OD2" s="1" t="inlineStr"/>
-      <c r="OE2" s="1" t="inlineStr"/>
-      <c r="OF2" s="1" t="inlineStr"/>
-      <c r="OG2" s="1" t="inlineStr"/>
-      <c r="OH2" s="1" t="inlineStr"/>
-      <c r="OI2" s="1" t="inlineStr"/>
-      <c r="OJ2" s="1" t="inlineStr"/>
-      <c r="OK2" s="1" t="inlineStr"/>
-      <c r="OL2" s="1" t="inlineStr"/>
-      <c r="OM2" s="1" t="inlineStr"/>
-      <c r="ON2" s="1" t="inlineStr"/>
-      <c r="OO2" s="1" t="inlineStr"/>
-      <c r="OP2" s="1" t="inlineStr"/>
-      <c r="OQ2" s="1" t="inlineStr"/>
-      <c r="OR2" s="1" t="inlineStr"/>
-      <c r="OS2" s="1" t="inlineStr"/>
-      <c r="OT2" s="1" t="inlineStr"/>
-      <c r="OU2" s="1" t="inlineStr"/>
-      <c r="OV2" s="1" t="inlineStr"/>
-      <c r="OW2" s="1" t="inlineStr"/>
-      <c r="OX2" s="1" t="inlineStr"/>
-      <c r="OY2" s="1" t="inlineStr"/>
-      <c r="OZ2" s="1" t="inlineStr"/>
-      <c r="PA2" s="1" t="inlineStr"/>
-      <c r="PB2" s="1" t="inlineStr"/>
-      <c r="PC2" s="1" t="inlineStr"/>
-      <c r="PD2" s="1" t="inlineStr"/>
-      <c r="PE2" s="1" t="inlineStr"/>
-      <c r="PF2" s="1" t="inlineStr"/>
-      <c r="PG2" s="1" t="inlineStr"/>
-      <c r="PH2" s="1" t="inlineStr"/>
-      <c r="PI2" s="1" t="inlineStr"/>
-      <c r="PJ2" s="1" t="inlineStr"/>
-      <c r="PK2" s="1" t="inlineStr"/>
-      <c r="PL2" s="1" t="inlineStr"/>
-      <c r="PM2" s="1" t="inlineStr"/>
-      <c r="PN2" s="1" t="inlineStr"/>
-      <c r="PO2" s="1" t="inlineStr"/>
-      <c r="PP2" s="1" t="inlineStr"/>
-      <c r="PQ2" s="1" t="inlineStr"/>
-      <c r="PR2" s="1" t="inlineStr"/>
-      <c r="PS2" s="1" t="inlineStr"/>
-      <c r="PT2" s="1" t="inlineStr"/>
-      <c r="PU2" s="1" t="inlineStr"/>
-      <c r="PV2" s="1" t="inlineStr"/>
-      <c r="PW2" s="1" t="inlineStr"/>
-      <c r="PX2" s="1" t="inlineStr"/>
-      <c r="PY2" s="1" t="inlineStr"/>
-      <c r="PZ2" s="1" t="inlineStr"/>
-      <c r="QA2" s="1" t="inlineStr"/>
-      <c r="QB2" s="1" t="inlineStr"/>
-      <c r="QC2" s="1" t="inlineStr"/>
-      <c r="QD2" s="1" t="inlineStr"/>
-      <c r="QE2" s="1" t="inlineStr"/>
-      <c r="QF2" s="1" t="inlineStr"/>
-      <c r="QG2" s="1" t="inlineStr"/>
-      <c r="QH2" s="1" t="inlineStr"/>
-      <c r="QI2" s="1" t="inlineStr"/>
-      <c r="QJ2" s="1" t="inlineStr"/>
-      <c r="QK2" s="1" t="inlineStr"/>
-      <c r="QL2" s="1" t="inlineStr"/>
-      <c r="QM2" s="1" t="inlineStr"/>
-      <c r="QN2" s="1" t="inlineStr"/>
-      <c r="QO2" s="1" t="inlineStr"/>
-      <c r="QP2" s="1" t="inlineStr"/>
-      <c r="QQ2" s="1" t="inlineStr"/>
-      <c r="QR2" s="1" t="inlineStr"/>
-      <c r="QS2" s="1" t="inlineStr"/>
-      <c r="QT2" s="1" t="inlineStr"/>
-      <c r="QU2" s="1" t="inlineStr"/>
-      <c r="QV2" s="1" t="inlineStr"/>
-      <c r="QW2" s="1" t="inlineStr"/>
+      <c r="B2" s="2" t="inlineStr"/>
+      <c r="C2" s="2" t="inlineStr"/>
+      <c r="D2" s="2" t="inlineStr"/>
+      <c r="E2" s="2" t="inlineStr"/>
+      <c r="F2" s="2" t="inlineStr"/>
+      <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr"/>
+      <c r="I2" s="2" t="inlineStr"/>
+      <c r="J2" s="2" t="inlineStr"/>
+      <c r="K2" s="2" t="inlineStr"/>
+      <c r="L2" s="2" t="inlineStr"/>
+      <c r="M2" s="2" t="inlineStr"/>
+      <c r="N2" s="2" t="inlineStr"/>
+      <c r="O2" s="2" t="inlineStr"/>
+      <c r="P2" s="2" t="inlineStr"/>
+      <c r="Q2" s="2" t="inlineStr"/>
+      <c r="R2" s="2" t="inlineStr"/>
+      <c r="S2" s="2" t="inlineStr"/>
+      <c r="T2" s="2" t="inlineStr"/>
+      <c r="U2" s="2" t="inlineStr"/>
+      <c r="V2" s="2" t="inlineStr"/>
+      <c r="W2" s="2" t="inlineStr"/>
+      <c r="X2" s="2" t="inlineStr"/>
+      <c r="Y2" s="2" t="inlineStr"/>
+      <c r="Z2" s="2" t="inlineStr"/>
+      <c r="AA2" s="2" t="inlineStr"/>
+      <c r="AB2" s="2" t="inlineStr"/>
+      <c r="AC2" s="2" t="inlineStr"/>
+      <c r="AD2" s="2" t="inlineStr"/>
+      <c r="AE2" s="2" t="inlineStr"/>
+      <c r="AF2" s="2" t="inlineStr"/>
+      <c r="AG2" s="2" t="inlineStr"/>
+      <c r="AH2" s="2" t="inlineStr"/>
+      <c r="AI2" s="2" t="inlineStr"/>
+      <c r="AJ2" s="2" t="inlineStr"/>
+      <c r="AK2" s="2" t="inlineStr"/>
+      <c r="AL2" s="2" t="inlineStr"/>
+      <c r="AM2" s="2" t="inlineStr"/>
+      <c r="AN2" s="2" t="inlineStr"/>
+      <c r="AO2" s="2" t="inlineStr"/>
+      <c r="AP2" s="2" t="inlineStr"/>
+      <c r="AQ2" s="2" t="inlineStr"/>
+      <c r="AR2" s="2" t="inlineStr"/>
+      <c r="AS2" s="2" t="inlineStr"/>
+      <c r="AT2" s="2" t="inlineStr"/>
+      <c r="AU2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AW2" s="2" t="inlineStr"/>
+      <c r="AX2" s="2" t="inlineStr"/>
+      <c r="AY2" s="2" t="inlineStr"/>
+      <c r="AZ2" s="2" t="inlineStr"/>
+      <c r="BA2" s="2" t="inlineStr"/>
+      <c r="BB2" s="2" t="inlineStr"/>
+      <c r="BC2" s="2" t="inlineStr"/>
+      <c r="BD2" s="2" t="inlineStr"/>
+      <c r="BE2" s="2" t="inlineStr"/>
+      <c r="BF2" s="2" t="inlineStr"/>
+      <c r="BG2" s="2" t="inlineStr"/>
+      <c r="BH2" s="2" t="inlineStr"/>
+      <c r="BI2" s="2" t="inlineStr"/>
+      <c r="BJ2" s="2" t="inlineStr"/>
+      <c r="BK2" s="2" t="inlineStr"/>
+      <c r="BL2" s="2" t="inlineStr"/>
+      <c r="BM2" s="2" t="inlineStr"/>
+      <c r="BN2" s="2" t="inlineStr"/>
+      <c r="BO2" s="2" t="inlineStr"/>
+      <c r="BP2" s="2" t="inlineStr"/>
+      <c r="BQ2" s="2" t="inlineStr"/>
+      <c r="BR2" s="2" t="inlineStr"/>
+      <c r="BS2" s="2" t="inlineStr"/>
+      <c r="BT2" s="2" t="inlineStr"/>
+      <c r="BU2" s="2" t="inlineStr"/>
+      <c r="BV2" s="2" t="inlineStr"/>
+      <c r="BW2" s="2" t="inlineStr"/>
+      <c r="BX2" s="2" t="inlineStr"/>
+      <c r="BY2" s="2" t="inlineStr"/>
+      <c r="BZ2" s="2" t="inlineStr"/>
+      <c r="CA2" s="2" t="inlineStr"/>
+      <c r="CB2" s="2" t="inlineStr"/>
+      <c r="CC2" s="2" t="inlineStr"/>
+      <c r="CD2" s="2" t="inlineStr"/>
+      <c r="CE2" s="2" t="inlineStr"/>
+      <c r="CF2" s="2" t="inlineStr"/>
+      <c r="CG2" s="2" t="inlineStr"/>
+      <c r="CH2" s="2" t="inlineStr"/>
+      <c r="CI2" s="2" t="inlineStr"/>
+      <c r="CJ2" s="2" t="inlineStr"/>
+      <c r="CK2" s="2" t="inlineStr"/>
+      <c r="CL2" s="2" t="inlineStr"/>
+      <c r="CM2" s="2" t="inlineStr"/>
+      <c r="CN2" s="2" t="inlineStr"/>
+      <c r="CO2" s="2" t="inlineStr"/>
+      <c r="CP2" s="2" t="inlineStr"/>
+      <c r="CQ2" s="2" t="inlineStr"/>
+      <c r="CR2" s="2" t="inlineStr"/>
+      <c r="CS2" s="2" t="inlineStr"/>
+      <c r="CT2" s="2" t="inlineStr"/>
+      <c r="CU2" s="2" t="inlineStr"/>
+      <c r="CV2" s="2" t="inlineStr"/>
+      <c r="CW2" s="2" t="inlineStr"/>
+      <c r="CX2" s="2" t="inlineStr"/>
+      <c r="CY2" s="2" t="inlineStr"/>
+      <c r="CZ2" s="2" t="inlineStr"/>
+      <c r="DA2" s="2" t="inlineStr"/>
+      <c r="DB2" s="2" t="inlineStr"/>
+      <c r="DC2" s="2" t="inlineStr"/>
+      <c r="DD2" s="2" t="inlineStr"/>
+      <c r="DE2" s="2" t="inlineStr"/>
+      <c r="DF2" s="2" t="inlineStr"/>
+      <c r="DG2" s="2" t="inlineStr"/>
+      <c r="DH2" s="2" t="inlineStr"/>
+      <c r="DI2" s="2" t="inlineStr"/>
+      <c r="DJ2" s="2" t="inlineStr"/>
+      <c r="DK2" s="2" t="inlineStr"/>
+      <c r="DL2" s="2" t="inlineStr"/>
+      <c r="DM2" s="2" t="inlineStr"/>
+      <c r="DN2" s="2" t="inlineStr"/>
+      <c r="DO2" s="2" t="inlineStr"/>
+      <c r="DP2" s="2" t="inlineStr"/>
+      <c r="DQ2" s="2" t="inlineStr"/>
+      <c r="DR2" s="2" t="inlineStr"/>
+      <c r="DS2" s="2" t="inlineStr"/>
+      <c r="DT2" s="2" t="inlineStr"/>
+      <c r="DU2" s="2" t="inlineStr"/>
+      <c r="DV2" s="2" t="inlineStr"/>
+      <c r="DW2" s="2" t="inlineStr"/>
+      <c r="DX2" s="2" t="inlineStr"/>
+      <c r="DY2" s="2" t="inlineStr"/>
+      <c r="DZ2" s="2" t="inlineStr"/>
+      <c r="EA2" s="2" t="inlineStr"/>
+      <c r="EB2" s="2" t="inlineStr"/>
+      <c r="EC2" s="2" t="inlineStr"/>
+      <c r="ED2" s="2" t="inlineStr"/>
+      <c r="EE2" s="2" t="inlineStr"/>
+      <c r="EF2" s="2" t="inlineStr"/>
+      <c r="EG2" s="2" t="inlineStr"/>
+      <c r="EH2" s="2" t="inlineStr"/>
+      <c r="EI2" s="2" t="inlineStr"/>
+      <c r="EJ2" s="2" t="inlineStr"/>
+      <c r="EK2" s="2" t="inlineStr"/>
+      <c r="EL2" s="2" t="inlineStr"/>
+      <c r="EM2" s="2" t="inlineStr"/>
+      <c r="EN2" s="2" t="inlineStr"/>
+      <c r="EO2" s="2" t="inlineStr"/>
+      <c r="EP2" s="2" t="inlineStr"/>
+      <c r="EQ2" s="2" t="inlineStr"/>
+      <c r="ER2" s="2" t="inlineStr"/>
+      <c r="ES2" s="2" t="inlineStr"/>
+      <c r="ET2" s="2" t="inlineStr"/>
+      <c r="EU2" s="2" t="inlineStr"/>
+      <c r="EV2" s="2" t="inlineStr"/>
+      <c r="EW2" s="2" t="inlineStr"/>
+      <c r="EX2" s="2" t="inlineStr"/>
+      <c r="EY2" s="2" t="inlineStr"/>
+      <c r="EZ2" s="2" t="inlineStr"/>
+      <c r="FA2" s="2" t="inlineStr"/>
+      <c r="FB2" s="2" t="inlineStr"/>
+      <c r="FC2" s="2" t="inlineStr"/>
+      <c r="FD2" s="2" t="inlineStr"/>
+      <c r="FE2" s="2" t="inlineStr"/>
+      <c r="FF2" s="2" t="inlineStr"/>
+      <c r="FG2" s="2" t="inlineStr"/>
+      <c r="FH2" s="2" t="inlineStr"/>
+      <c r="FI2" s="2" t="inlineStr"/>
+      <c r="FJ2" s="2" t="inlineStr"/>
+      <c r="FK2" s="2" t="inlineStr"/>
+      <c r="FL2" s="2" t="inlineStr"/>
+      <c r="FM2" s="2" t="inlineStr"/>
+      <c r="FN2" s="2" t="inlineStr"/>
+      <c r="FO2" s="2" t="inlineStr"/>
+      <c r="FP2" s="2" t="inlineStr"/>
+      <c r="FQ2" s="2" t="inlineStr"/>
+      <c r="FR2" s="2" t="inlineStr"/>
+      <c r="FS2" s="2" t="inlineStr"/>
+      <c r="FT2" s="2" t="inlineStr"/>
+      <c r="FU2" s="2" t="inlineStr"/>
+      <c r="FV2" s="2" t="inlineStr"/>
+      <c r="FW2" s="2" t="inlineStr"/>
+      <c r="FX2" s="2" t="inlineStr"/>
+      <c r="FY2" s="2" t="inlineStr"/>
+      <c r="FZ2" s="2" t="inlineStr"/>
+      <c r="GA2" s="2" t="inlineStr"/>
+      <c r="GB2" s="2" t="inlineStr"/>
+      <c r="GC2" s="2" t="inlineStr"/>
+      <c r="GD2" s="2" t="inlineStr"/>
+      <c r="GE2" s="2" t="inlineStr"/>
+      <c r="GF2" s="2" t="inlineStr"/>
+      <c r="GG2" s="2" t="inlineStr"/>
+      <c r="GH2" s="2" t="inlineStr"/>
+      <c r="GI2" s="2" t="inlineStr"/>
+      <c r="GJ2" s="2" t="inlineStr"/>
+      <c r="GK2" s="2" t="inlineStr"/>
+      <c r="GL2" s="2" t="inlineStr"/>
+      <c r="GM2" s="2" t="inlineStr"/>
+      <c r="GN2" s="2" t="inlineStr"/>
+      <c r="GO2" s="2" t="inlineStr"/>
+      <c r="GP2" s="2" t="inlineStr"/>
+      <c r="GQ2" s="2" t="inlineStr"/>
+      <c r="GR2" s="2" t="inlineStr"/>
+      <c r="GS2" s="2" t="inlineStr"/>
+      <c r="GT2" s="2" t="inlineStr"/>
+      <c r="GU2" s="2" t="inlineStr"/>
+      <c r="GV2" s="2" t="inlineStr"/>
+      <c r="GW2" s="2" t="inlineStr"/>
+      <c r="GX2" s="2" t="inlineStr"/>
+      <c r="GY2" s="2" t="inlineStr"/>
+      <c r="GZ2" s="2" t="inlineStr"/>
+      <c r="HA2" s="2" t="inlineStr"/>
+      <c r="HB2" s="2" t="inlineStr"/>
+      <c r="HC2" s="2" t="inlineStr"/>
+      <c r="HD2" s="2" t="inlineStr"/>
+      <c r="HE2" s="2" t="inlineStr"/>
+      <c r="HF2" s="2" t="inlineStr"/>
+      <c r="HG2" s="2" t="inlineStr"/>
+      <c r="HH2" s="2" t="inlineStr"/>
+      <c r="HI2" s="2" t="inlineStr"/>
+      <c r="HJ2" s="2" t="inlineStr"/>
+      <c r="HK2" s="2" t="inlineStr"/>
+      <c r="HL2" s="2" t="inlineStr"/>
+      <c r="HM2" s="2" t="inlineStr"/>
+      <c r="HN2" s="2" t="inlineStr"/>
+      <c r="HO2" s="2" t="inlineStr"/>
+      <c r="HP2" s="2" t="inlineStr"/>
+      <c r="HQ2" s="2" t="inlineStr"/>
+      <c r="HR2" s="2" t="inlineStr"/>
+      <c r="HS2" s="2" t="inlineStr"/>
+      <c r="HT2" s="2" t="inlineStr"/>
+      <c r="HU2" s="2" t="inlineStr"/>
+      <c r="HV2" s="2" t="inlineStr"/>
+      <c r="HW2" s="2" t="inlineStr"/>
+      <c r="HX2" s="2" t="inlineStr"/>
+      <c r="HY2" s="2" t="inlineStr"/>
+      <c r="HZ2" s="2" t="inlineStr"/>
+      <c r="IA2" s="2" t="inlineStr"/>
+      <c r="IB2" s="2" t="inlineStr"/>
+      <c r="IC2" s="2" t="inlineStr"/>
+      <c r="ID2" s="2" t="inlineStr"/>
+      <c r="IE2" s="2" t="inlineStr"/>
+      <c r="IF2" s="2" t="inlineStr"/>
+      <c r="IG2" s="2" t="inlineStr"/>
+      <c r="IH2" s="2" t="inlineStr"/>
+      <c r="II2" s="2" t="inlineStr"/>
+      <c r="IJ2" s="2" t="inlineStr"/>
+      <c r="IK2" s="2" t="inlineStr"/>
+      <c r="IL2" s="2" t="inlineStr"/>
+      <c r="IM2" s="2" t="inlineStr"/>
+      <c r="IN2" s="2" t="inlineStr"/>
+      <c r="IO2" s="2" t="inlineStr"/>
+      <c r="IP2" s="2" t="inlineStr"/>
+      <c r="IQ2" s="2" t="inlineStr"/>
+      <c r="IR2" s="2" t="inlineStr"/>
+      <c r="IS2" s="2" t="inlineStr"/>
+      <c r="IT2" s="2" t="inlineStr"/>
+      <c r="IU2" s="2" t="inlineStr"/>
+      <c r="IV2" s="2" t="inlineStr"/>
+      <c r="IW2" s="2" t="inlineStr"/>
+      <c r="IX2" s="2" t="inlineStr"/>
+      <c r="IY2" s="2" t="inlineStr"/>
+      <c r="IZ2" s="2" t="inlineStr"/>
+      <c r="JA2" s="2" t="inlineStr"/>
+      <c r="JB2" s="2" t="inlineStr"/>
+      <c r="JC2" s="2" t="inlineStr"/>
+      <c r="JD2" s="2" t="inlineStr"/>
+      <c r="JE2" s="2" t="inlineStr"/>
+      <c r="JF2" s="2" t="inlineStr"/>
+      <c r="JG2" s="2" t="inlineStr"/>
+      <c r="JH2" s="2" t="inlineStr"/>
+      <c r="JI2" s="2" t="inlineStr"/>
+      <c r="JJ2" s="2" t="inlineStr"/>
+      <c r="JK2" s="2" t="inlineStr"/>
+      <c r="JL2" s="2" t="inlineStr"/>
+      <c r="JM2" s="2" t="inlineStr"/>
+      <c r="JN2" s="2" t="inlineStr"/>
+      <c r="JO2" s="2" t="inlineStr"/>
+      <c r="JP2" s="2" t="inlineStr"/>
+      <c r="JQ2" s="2" t="inlineStr"/>
+      <c r="JR2" s="2" t="inlineStr"/>
+      <c r="JS2" s="2" t="inlineStr"/>
+      <c r="JT2" s="2" t="inlineStr"/>
+      <c r="JU2" s="2" t="inlineStr"/>
+      <c r="JV2" s="2" t="inlineStr"/>
+      <c r="JW2" s="2" t="inlineStr"/>
+      <c r="JX2" s="2" t="inlineStr"/>
+      <c r="JY2" s="2" t="inlineStr"/>
+      <c r="JZ2" s="2" t="inlineStr"/>
+      <c r="KA2" s="2" t="inlineStr"/>
+      <c r="KB2" s="2" t="inlineStr"/>
+      <c r="KC2" s="2" t="inlineStr"/>
+      <c r="KD2" s="2" t="inlineStr"/>
+      <c r="KE2" s="2" t="inlineStr"/>
+      <c r="KF2" s="2" t="inlineStr"/>
+      <c r="KG2" s="2" t="inlineStr"/>
+      <c r="KH2" s="2" t="inlineStr"/>
+      <c r="KI2" s="2" t="inlineStr"/>
+      <c r="KJ2" s="2" t="inlineStr"/>
+      <c r="KK2" s="2" t="inlineStr"/>
+      <c r="KL2" s="2" t="inlineStr"/>
+      <c r="KM2" s="2" t="inlineStr"/>
+      <c r="KN2" s="2" t="inlineStr"/>
+      <c r="KO2" s="2" t="inlineStr"/>
+      <c r="KP2" s="2" t="inlineStr"/>
+      <c r="KQ2" s="2" t="inlineStr"/>
+      <c r="KR2" s="2" t="inlineStr"/>
+      <c r="KS2" s="2" t="inlineStr"/>
+      <c r="KT2" s="2" t="inlineStr"/>
+      <c r="KU2" s="2" t="inlineStr"/>
+      <c r="KV2" s="2" t="inlineStr"/>
+      <c r="KW2" s="2" t="inlineStr"/>
+      <c r="KX2" s="2" t="inlineStr"/>
+      <c r="KY2" s="2" t="inlineStr"/>
+      <c r="KZ2" s="2" t="inlineStr"/>
+      <c r="LA2" s="2" t="inlineStr"/>
+      <c r="LB2" s="2" t="inlineStr"/>
+      <c r="LC2" s="2" t="inlineStr"/>
+      <c r="LD2" s="2" t="inlineStr"/>
+      <c r="LE2" s="2" t="inlineStr"/>
+      <c r="LF2" s="2" t="inlineStr"/>
+      <c r="LG2" s="2" t="inlineStr"/>
+      <c r="LH2" s="2" t="inlineStr"/>
+      <c r="LI2" s="2" t="inlineStr"/>
+      <c r="LJ2" s="2" t="inlineStr"/>
+      <c r="LK2" s="2" t="inlineStr"/>
+      <c r="LL2" s="2" t="inlineStr"/>
+      <c r="LM2" s="2" t="inlineStr"/>
+      <c r="LN2" s="2" t="inlineStr"/>
+      <c r="LO2" s="2" t="inlineStr"/>
+      <c r="LP2" s="2" t="inlineStr"/>
+      <c r="LQ2" s="2" t="inlineStr"/>
+      <c r="LR2" s="2" t="inlineStr"/>
+      <c r="LS2" s="2" t="inlineStr"/>
+      <c r="LT2" s="2" t="inlineStr"/>
+      <c r="LU2" s="2" t="inlineStr"/>
+      <c r="LV2" s="2" t="inlineStr"/>
+      <c r="LW2" s="2" t="inlineStr"/>
+      <c r="LX2" s="2" t="inlineStr"/>
+      <c r="LY2" s="2" t="inlineStr"/>
+      <c r="LZ2" s="2" t="inlineStr"/>
+      <c r="MA2" s="2" t="inlineStr"/>
+      <c r="MB2" s="2" t="inlineStr"/>
+      <c r="MC2" s="2" t="inlineStr"/>
+      <c r="MD2" s="2" t="inlineStr"/>
+      <c r="ME2" s="2" t="inlineStr"/>
+      <c r="MF2" s="2" t="inlineStr"/>
+      <c r="MG2" s="2" t="inlineStr"/>
+      <c r="MH2" s="2" t="inlineStr"/>
+      <c r="MI2" s="2" t="inlineStr"/>
+      <c r="MJ2" s="2" t="inlineStr"/>
+      <c r="MK2" s="2" t="inlineStr"/>
+      <c r="ML2" s="2" t="inlineStr"/>
+      <c r="MM2" s="2" t="inlineStr"/>
+      <c r="MN2" s="2" t="inlineStr"/>
+      <c r="MO2" s="2" t="inlineStr"/>
+      <c r="MP2" s="2" t="inlineStr"/>
+      <c r="MQ2" s="2" t="inlineStr"/>
+      <c r="MR2" s="2" t="inlineStr"/>
+      <c r="MS2" s="2" t="inlineStr"/>
+      <c r="MT2" s="2" t="inlineStr"/>
+      <c r="MU2" s="2" t="inlineStr"/>
+      <c r="MV2" s="2" t="inlineStr"/>
+      <c r="MW2" s="2" t="inlineStr"/>
+      <c r="MX2" s="2" t="inlineStr"/>
+      <c r="MY2" s="2" t="inlineStr"/>
+      <c r="MZ2" s="2" t="inlineStr"/>
+      <c r="NA2" s="2" t="inlineStr"/>
+      <c r="NB2" s="2" t="inlineStr"/>
+      <c r="NC2" s="2" t="inlineStr"/>
+      <c r="ND2" s="2" t="inlineStr"/>
+      <c r="NE2" s="2" t="inlineStr"/>
+      <c r="NF2" s="2" t="inlineStr"/>
+      <c r="NG2" s="2" t="inlineStr"/>
+      <c r="NH2" s="2" t="inlineStr"/>
+      <c r="NI2" s="2" t="inlineStr"/>
+      <c r="NJ2" s="2" t="inlineStr"/>
+      <c r="NK2" s="2" t="inlineStr"/>
+      <c r="NL2" s="2" t="inlineStr"/>
+      <c r="NM2" s="2" t="inlineStr"/>
+      <c r="NN2" s="2" t="inlineStr"/>
+      <c r="NO2" s="2" t="inlineStr"/>
+      <c r="NP2" s="2" t="inlineStr"/>
+      <c r="NQ2" s="2" t="inlineStr"/>
+      <c r="NR2" s="2" t="inlineStr"/>
+      <c r="NS2" s="2" t="inlineStr"/>
+      <c r="NT2" s="2" t="inlineStr"/>
+      <c r="NU2" s="2" t="inlineStr"/>
+      <c r="NV2" s="2" t="inlineStr"/>
+      <c r="NW2" s="2" t="inlineStr"/>
+      <c r="NX2" s="2" t="inlineStr"/>
+      <c r="NY2" s="2" t="inlineStr"/>
+      <c r="NZ2" s="2" t="inlineStr"/>
+      <c r="OA2" s="2" t="inlineStr"/>
+      <c r="OB2" s="2" t="inlineStr"/>
+      <c r="OC2" s="2" t="inlineStr"/>
+      <c r="OD2" s="2" t="inlineStr"/>
+      <c r="OE2" s="2" t="inlineStr"/>
+      <c r="OF2" s="2" t="inlineStr"/>
+      <c r="OG2" s="2" t="inlineStr"/>
+      <c r="OH2" s="2" t="inlineStr"/>
+      <c r="OI2" s="2" t="inlineStr"/>
+      <c r="OJ2" s="2" t="inlineStr"/>
+      <c r="OK2" s="2" t="inlineStr"/>
+      <c r="OL2" s="2" t="inlineStr"/>
+      <c r="OM2" s="2" t="inlineStr"/>
+      <c r="ON2" s="2" t="inlineStr"/>
+      <c r="OO2" s="2" t="inlineStr"/>
+      <c r="OP2" s="2" t="inlineStr"/>
+      <c r="OQ2" s="2" t="inlineStr"/>
+      <c r="OR2" s="2" t="inlineStr"/>
+      <c r="OS2" s="2" t="inlineStr"/>
+      <c r="OT2" s="2" t="inlineStr"/>
+      <c r="OU2" s="2" t="inlineStr"/>
+      <c r="OV2" s="2" t="inlineStr"/>
+      <c r="OW2" s="2" t="inlineStr"/>
+      <c r="OX2" s="2" t="inlineStr"/>
+      <c r="OY2" s="2" t="inlineStr"/>
+      <c r="OZ2" s="2" t="inlineStr"/>
+      <c r="PA2" s="2" t="inlineStr"/>
+      <c r="PB2" s="2" t="inlineStr"/>
+      <c r="PC2" s="2" t="inlineStr"/>
+      <c r="PD2" s="2" t="inlineStr"/>
+      <c r="PE2" s="2" t="inlineStr"/>
+      <c r="PF2" s="2" t="inlineStr"/>
+      <c r="PG2" s="2" t="inlineStr"/>
+      <c r="PH2" s="2" t="inlineStr"/>
+      <c r="PI2" s="2" t="inlineStr"/>
+      <c r="PJ2" s="2" t="inlineStr"/>
+      <c r="PK2" s="2" t="inlineStr"/>
+      <c r="PL2" s="2" t="inlineStr"/>
+      <c r="PM2" s="2" t="inlineStr"/>
+      <c r="PN2" s="2" t="inlineStr"/>
+      <c r="PO2" s="2" t="inlineStr"/>
+      <c r="PP2" s="2" t="inlineStr"/>
+      <c r="PQ2" s="2" t="inlineStr"/>
+      <c r="PR2" s="2" t="inlineStr"/>
+      <c r="PS2" s="2" t="inlineStr"/>
+      <c r="PT2" s="2" t="inlineStr"/>
+      <c r="PU2" s="2" t="inlineStr"/>
+      <c r="PV2" s="2" t="inlineStr"/>
+      <c r="PW2" s="2" t="inlineStr"/>
+      <c r="PX2" s="2" t="inlineStr"/>
+      <c r="PY2" s="2" t="inlineStr"/>
+      <c r="PZ2" s="2" t="inlineStr"/>
+      <c r="QA2" s="2" t="inlineStr"/>
+      <c r="QB2" s="2" t="inlineStr"/>
+      <c r="QC2" s="2" t="inlineStr"/>
+      <c r="QD2" s="2" t="inlineStr"/>
+      <c r="QE2" s="2" t="inlineStr"/>
+      <c r="QF2" s="2" t="inlineStr"/>
+      <c r="QG2" s="2" t="inlineStr"/>
+      <c r="QH2" s="2" t="inlineStr"/>
+      <c r="QI2" s="2" t="inlineStr"/>
+      <c r="QJ2" s="2" t="inlineStr"/>
+      <c r="QK2" s="2" t="inlineStr"/>
+      <c r="QL2" s="2" t="inlineStr"/>
+      <c r="QM2" s="2" t="inlineStr"/>
+      <c r="QN2" s="2" t="inlineStr"/>
+      <c r="QO2" s="2" t="inlineStr"/>
+      <c r="QP2" s="2" t="inlineStr"/>
+      <c r="QQ2" s="2" t="inlineStr"/>
+      <c r="QR2" s="2" t="inlineStr"/>
+      <c r="QS2" s="2" t="inlineStr"/>
+      <c r="QT2" s="2" t="inlineStr"/>
+      <c r="QU2" s="2" t="inlineStr"/>
+      <c r="QV2" s="2" t="inlineStr"/>
+      <c r="QW2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>2026-04-25</t>
         </is>
       </c>
-      <c r="B3" s="1" t="inlineStr"/>
-      <c r="C3" s="1" t="inlineStr"/>
-      <c r="D3" s="1" t="inlineStr"/>
-      <c r="E3" s="1" t="inlineStr"/>
-      <c r="F3" s="1" t="inlineStr"/>
-      <c r="G3" s="1" t="inlineStr"/>
-      <c r="H3" s="1" t="inlineStr"/>
-      <c r="I3" s="1" t="inlineStr"/>
-      <c r="J3" s="1" t="inlineStr"/>
-      <c r="K3" s="1" t="inlineStr"/>
-      <c r="L3" s="1" t="inlineStr"/>
-      <c r="M3" s="1" t="inlineStr"/>
-      <c r="N3" s="1" t="inlineStr"/>
-      <c r="O3" s="1" t="inlineStr"/>
-      <c r="P3" s="1" t="inlineStr"/>
-      <c r="Q3" s="1" t="inlineStr"/>
-      <c r="R3" s="1" t="inlineStr"/>
-      <c r="S3" s="1" t="inlineStr"/>
-      <c r="T3" s="1" t="inlineStr"/>
-      <c r="U3" s="1" t="inlineStr"/>
-      <c r="V3" s="1" t="inlineStr"/>
-      <c r="W3" s="1" t="inlineStr"/>
-      <c r="X3" s="1" t="inlineStr"/>
-      <c r="Y3" s="1" t="inlineStr"/>
-      <c r="Z3" s="1" t="inlineStr"/>
-      <c r="AA3" s="1" t="inlineStr"/>
-      <c r="AB3" s="1" t="inlineStr"/>
-      <c r="AC3" s="1" t="inlineStr"/>
-      <c r="AD3" s="1" t="inlineStr"/>
-      <c r="AE3" s="1" t="inlineStr"/>
-      <c r="AF3" s="1" t="inlineStr"/>
-      <c r="AG3" s="1" t="inlineStr"/>
-      <c r="AH3" s="1" t="inlineStr"/>
-      <c r="AI3" s="1" t="inlineStr"/>
-      <c r="AJ3" s="1" t="inlineStr"/>
-      <c r="AK3" s="1" t="inlineStr"/>
-      <c r="AL3" s="1" t="inlineStr"/>
-      <c r="AM3" s="1" t="inlineStr"/>
-      <c r="AN3" s="1" t="inlineStr"/>
-      <c r="AO3" s="1" t="inlineStr"/>
-      <c r="AP3" s="1" t="inlineStr"/>
-      <c r="AQ3" s="1" t="inlineStr"/>
-      <c r="AR3" s="1" t="inlineStr"/>
-      <c r="AS3" s="1" t="inlineStr"/>
-      <c r="AT3" s="1" t="inlineStr"/>
-      <c r="AU3" s="1" t="inlineStr"/>
-      <c r="AV3" s="1" t="inlineStr"/>
-      <c r="AW3" s="1" t="inlineStr"/>
-      <c r="AX3" s="1" t="inlineStr"/>
-      <c r="AY3" s="1" t="inlineStr"/>
-      <c r="AZ3" s="1" t="inlineStr"/>
-      <c r="BA3" s="1" t="inlineStr"/>
-      <c r="BB3" s="1" t="inlineStr"/>
-      <c r="BC3" s="1" t="inlineStr"/>
-      <c r="BD3" s="1" t="inlineStr"/>
-      <c r="BE3" s="1" t="inlineStr"/>
-      <c r="BF3" s="1" t="inlineStr"/>
-      <c r="BG3" s="1" t="inlineStr"/>
-      <c r="BH3" s="1" t="inlineStr"/>
-      <c r="BI3" s="1" t="inlineStr"/>
-      <c r="BJ3" s="1" t="inlineStr"/>
-      <c r="BK3" s="1" t="inlineStr"/>
-      <c r="BL3" s="1" t="inlineStr"/>
-      <c r="BM3" s="1" t="inlineStr"/>
-      <c r="BN3" s="1" t="inlineStr"/>
-      <c r="BO3" s="1" t="inlineStr"/>
-      <c r="BP3" s="1" t="inlineStr"/>
-      <c r="BQ3" s="1" t="inlineStr"/>
-      <c r="BR3" s="1" t="inlineStr"/>
-      <c r="BS3" s="1" t="inlineStr"/>
-      <c r="BT3" s="1" t="inlineStr"/>
-      <c r="BU3" s="1" t="inlineStr"/>
-      <c r="BV3" s="1" t="inlineStr"/>
-      <c r="BW3" s="1" t="inlineStr"/>
-      <c r="BX3" s="1" t="inlineStr"/>
-      <c r="BY3" s="1" t="inlineStr"/>
-      <c r="BZ3" s="1" t="inlineStr"/>
-      <c r="CA3" s="1" t="inlineStr"/>
-      <c r="CB3" s="1" t="inlineStr"/>
-      <c r="CC3" s="1" t="inlineStr"/>
-      <c r="CD3" s="1" t="inlineStr"/>
-      <c r="CE3" s="1" t="inlineStr"/>
-      <c r="CF3" s="1" t="inlineStr"/>
-      <c r="CG3" s="1" t="inlineStr"/>
-      <c r="CH3" s="1" t="inlineStr"/>
-      <c r="CI3" s="1" t="inlineStr"/>
-      <c r="CJ3" s="1" t="inlineStr"/>
-      <c r="CK3" s="1" t="inlineStr"/>
-      <c r="CL3" s="1" t="inlineStr"/>
-      <c r="CM3" s="1" t="inlineStr"/>
-      <c r="CN3" s="1" t="inlineStr"/>
-      <c r="CO3" s="1" t="inlineStr"/>
-      <c r="CP3" s="1" t="inlineStr"/>
-      <c r="CQ3" s="1" t="inlineStr"/>
-      <c r="CR3" s="1" t="inlineStr"/>
-      <c r="CS3" s="1" t="inlineStr"/>
-      <c r="CT3" s="1" t="inlineStr"/>
-      <c r="CU3" s="1" t="inlineStr"/>
-      <c r="CV3" s="1" t="inlineStr"/>
-      <c r="CW3" s="1" t="inlineStr"/>
-      <c r="CX3" s="1" t="inlineStr"/>
-      <c r="CY3" s="1" t="inlineStr"/>
-      <c r="CZ3" s="1" t="inlineStr"/>
-      <c r="DA3" s="1" t="inlineStr"/>
-      <c r="DB3" s="1" t="inlineStr"/>
-      <c r="DC3" s="1" t="inlineStr"/>
-      <c r="DD3" s="1" t="inlineStr"/>
-      <c r="DE3" s="1" t="inlineStr"/>
-      <c r="DF3" s="1" t="inlineStr"/>
-      <c r="DG3" s="1" t="inlineStr"/>
-      <c r="DH3" s="1" t="inlineStr"/>
-      <c r="DI3" s="1" t="inlineStr"/>
-      <c r="DJ3" s="1" t="inlineStr"/>
-      <c r="DK3" s="1" t="inlineStr"/>
-      <c r="DL3" s="1" t="inlineStr"/>
-      <c r="DM3" s="1" t="inlineStr"/>
-      <c r="DN3" s="1" t="inlineStr"/>
-      <c r="DO3" s="1" t="inlineStr"/>
-      <c r="DP3" s="1" t="inlineStr"/>
-      <c r="DQ3" s="1" t="inlineStr"/>
-      <c r="DR3" s="1" t="inlineStr"/>
-      <c r="DS3" s="1" t="inlineStr"/>
-      <c r="DT3" s="1" t="inlineStr"/>
-      <c r="DU3" s="1" t="inlineStr"/>
-      <c r="DV3" s="1" t="inlineStr"/>
-      <c r="DW3" s="1" t="inlineStr"/>
-      <c r="DX3" s="1" t="inlineStr"/>
-      <c r="DY3" s="1" t="inlineStr"/>
-      <c r="DZ3" s="1" t="inlineStr"/>
-      <c r="EA3" s="1" t="inlineStr"/>
-      <c r="EB3" s="1" t="inlineStr"/>
-      <c r="EC3" s="1" t="inlineStr"/>
-      <c r="ED3" s="1" t="inlineStr"/>
-      <c r="EE3" s="1" t="inlineStr"/>
-      <c r="EF3" s="1" t="inlineStr"/>
-      <c r="EG3" s="1" t="inlineStr"/>
-      <c r="EH3" s="1" t="inlineStr"/>
-      <c r="EI3" s="1" t="inlineStr"/>
-      <c r="EJ3" s="1" t="inlineStr"/>
-      <c r="EK3" s="1" t="inlineStr"/>
-      <c r="EL3" s="1" t="inlineStr"/>
-      <c r="EM3" s="1" t="inlineStr"/>
-      <c r="EN3" s="1" t="inlineStr"/>
-      <c r="EO3" s="1" t="inlineStr"/>
-      <c r="EP3" s="1" t="inlineStr"/>
-      <c r="EQ3" s="1" t="inlineStr"/>
-      <c r="ER3" s="1" t="inlineStr"/>
-      <c r="ES3" s="1" t="inlineStr"/>
-      <c r="ET3" s="1" t="inlineStr"/>
-      <c r="EU3" s="1" t="inlineStr"/>
-      <c r="EV3" s="1" t="inlineStr"/>
-      <c r="EW3" s="1" t="inlineStr"/>
-      <c r="EX3" s="1" t="inlineStr"/>
-      <c r="EY3" s="1" t="inlineStr"/>
-      <c r="EZ3" s="1" t="inlineStr"/>
-      <c r="FA3" s="1" t="inlineStr"/>
-      <c r="FB3" s="1" t="inlineStr"/>
-      <c r="FC3" s="1" t="inlineStr"/>
-      <c r="FD3" s="1" t="inlineStr"/>
-      <c r="FE3" s="1" t="inlineStr"/>
-      <c r="FF3" s="1" t="inlineStr"/>
-      <c r="FG3" s="1" t="inlineStr"/>
-      <c r="FH3" s="1" t="inlineStr"/>
-      <c r="FI3" s="1" t="inlineStr"/>
-      <c r="FJ3" s="1" t="inlineStr"/>
-      <c r="FK3" s="1" t="inlineStr"/>
-      <c r="FL3" s="1" t="inlineStr"/>
-      <c r="FM3" s="1" t="inlineStr"/>
-      <c r="FN3" s="1" t="inlineStr"/>
-      <c r="FO3" s="1" t="inlineStr"/>
-      <c r="FP3" s="1" t="inlineStr"/>
-      <c r="FQ3" s="1" t="inlineStr"/>
-      <c r="FR3" s="1" t="inlineStr"/>
-      <c r="FS3" s="1" t="inlineStr"/>
-      <c r="FT3" s="1" t="inlineStr"/>
-      <c r="FU3" s="1" t="inlineStr"/>
-      <c r="FV3" s="1" t="inlineStr"/>
-      <c r="FW3" s="1" t="inlineStr"/>
-      <c r="FX3" s="1" t="inlineStr"/>
-      <c r="FY3" s="1" t="inlineStr"/>
-      <c r="FZ3" s="1" t="inlineStr"/>
-      <c r="GA3" s="1" t="inlineStr"/>
-      <c r="GB3" s="1" t="inlineStr"/>
-      <c r="GC3" s="1" t="inlineStr"/>
-      <c r="GD3" s="1" t="inlineStr"/>
-      <c r="GE3" s="1" t="inlineStr"/>
-      <c r="GF3" s="1" t="inlineStr"/>
-      <c r="GG3" s="1" t="inlineStr"/>
-      <c r="GH3" s="1" t="inlineStr"/>
-      <c r="GI3" s="1" t="inlineStr"/>
-      <c r="GJ3" s="1" t="inlineStr"/>
-      <c r="GK3" s="1" t="inlineStr"/>
-      <c r="GL3" s="1" t="inlineStr"/>
-      <c r="GM3" s="1" t="inlineStr"/>
-      <c r="GN3" s="1" t="inlineStr"/>
-      <c r="GO3" s="1" t="inlineStr"/>
-      <c r="GP3" s="1" t="inlineStr"/>
-      <c r="GQ3" s="1" t="inlineStr"/>
-      <c r="GR3" s="1" t="inlineStr"/>
-      <c r="GS3" s="1" t="inlineStr"/>
-      <c r="GT3" s="1" t="inlineStr"/>
-      <c r="GU3" s="1" t="inlineStr"/>
-      <c r="GV3" s="1" t="inlineStr"/>
-      <c r="GW3" s="1" t="inlineStr"/>
-      <c r="GX3" s="1" t="inlineStr"/>
-      <c r="GY3" s="1" t="inlineStr"/>
-      <c r="GZ3" s="1" t="inlineStr"/>
-      <c r="HA3" s="1" t="inlineStr"/>
-      <c r="HB3" s="1" t="inlineStr"/>
-      <c r="HC3" s="1" t="inlineStr"/>
-      <c r="HD3" s="1" t="inlineStr"/>
-      <c r="HE3" s="1" t="inlineStr"/>
-      <c r="HF3" s="1" t="inlineStr"/>
-      <c r="HG3" s="1" t="inlineStr"/>
-      <c r="HH3" s="1" t="inlineStr"/>
-      <c r="HI3" s="1" t="inlineStr"/>
-      <c r="HJ3" s="1" t="inlineStr"/>
-      <c r="HK3" s="1" t="inlineStr"/>
-      <c r="HL3" s="1" t="inlineStr"/>
-      <c r="HM3" s="1" t="inlineStr"/>
-      <c r="HN3" s="1" t="inlineStr"/>
-      <c r="HO3" s="1" t="inlineStr"/>
-      <c r="HP3" s="1" t="inlineStr"/>
-      <c r="HQ3" s="1" t="inlineStr"/>
-      <c r="HR3" s="1" t="inlineStr"/>
-      <c r="HS3" s="1" t="inlineStr"/>
-      <c r="HT3" s="1" t="inlineStr"/>
-      <c r="HU3" s="1" t="inlineStr"/>
-      <c r="HV3" s="1" t="inlineStr"/>
-      <c r="HW3" s="1" t="inlineStr"/>
-      <c r="HX3" s="1" t="inlineStr"/>
-      <c r="HY3" s="1" t="inlineStr"/>
-      <c r="HZ3" s="1" t="inlineStr"/>
-      <c r="IA3" s="1" t="inlineStr"/>
-      <c r="IB3" s="1" t="inlineStr"/>
-      <c r="IC3" s="1" t="inlineStr"/>
-      <c r="ID3" s="1" t="inlineStr"/>
-      <c r="IE3" s="1" t="inlineStr"/>
-      <c r="IF3" s="1" t="inlineStr"/>
-      <c r="IG3" s="1" t="inlineStr"/>
-      <c r="IH3" s="1" t="inlineStr"/>
-      <c r="II3" s="1" t="inlineStr"/>
-      <c r="IJ3" s="1" t="inlineStr"/>
-      <c r="IK3" s="1" t="inlineStr"/>
-      <c r="IL3" s="1" t="inlineStr"/>
-      <c r="IM3" s="1" t="inlineStr"/>
-      <c r="IN3" s="1" t="inlineStr"/>
-      <c r="IO3" s="1" t="inlineStr"/>
-      <c r="IP3" s="1" t="inlineStr"/>
-      <c r="IQ3" s="1" t="inlineStr"/>
-      <c r="IR3" s="1" t="inlineStr"/>
-      <c r="IS3" s="1" t="inlineStr"/>
-      <c r="IT3" s="1" t="inlineStr"/>
-      <c r="IU3" s="1" t="inlineStr"/>
-      <c r="IV3" s="1" t="inlineStr"/>
-      <c r="IW3" s="1" t="inlineStr"/>
-      <c r="IX3" s="1" t="inlineStr"/>
-      <c r="IY3" s="1" t="inlineStr"/>
-      <c r="IZ3" s="1" t="inlineStr"/>
-      <c r="JA3" s="1" t="inlineStr"/>
-      <c r="JB3" s="1" t="inlineStr"/>
-      <c r="JC3" s="1" t="inlineStr"/>
-      <c r="JD3" s="1" t="inlineStr"/>
-      <c r="JE3" s="1" t="inlineStr"/>
-      <c r="JF3" s="1" t="inlineStr"/>
-      <c r="JG3" s="1" t="inlineStr"/>
-      <c r="JH3" s="1" t="inlineStr"/>
-      <c r="JI3" s="1" t="inlineStr"/>
-      <c r="JJ3" s="1" t="inlineStr"/>
-      <c r="JK3" s="1" t="inlineStr"/>
-      <c r="JL3" s="1" t="inlineStr"/>
-      <c r="JM3" s="1" t="inlineStr"/>
-      <c r="JN3" s="1" t="inlineStr"/>
-      <c r="JO3" s="1" t="inlineStr"/>
-      <c r="JP3" s="1" t="inlineStr"/>
-      <c r="JQ3" s="1" t="inlineStr"/>
-      <c r="JR3" s="1" t="inlineStr"/>
-      <c r="JS3" s="1" t="inlineStr"/>
-      <c r="JT3" s="1" t="inlineStr"/>
-      <c r="JU3" s="1" t="inlineStr"/>
-      <c r="JV3" s="1" t="inlineStr"/>
-      <c r="JW3" s="1" t="inlineStr"/>
-      <c r="JX3" s="1" t="inlineStr"/>
-      <c r="JY3" s="1" t="inlineStr"/>
-      <c r="JZ3" s="1" t="inlineStr"/>
-      <c r="KA3" s="1" t="inlineStr"/>
-      <c r="KB3" s="1" t="inlineStr"/>
-      <c r="KC3" s="1" t="inlineStr"/>
-      <c r="KD3" s="1" t="inlineStr"/>
-      <c r="KE3" s="1" t="inlineStr"/>
-      <c r="KF3" s="1" t="inlineStr"/>
-      <c r="KG3" s="1" t="inlineStr"/>
-      <c r="KH3" s="1" t="inlineStr"/>
-      <c r="KI3" s="1" t="inlineStr"/>
-      <c r="KJ3" s="1" t="inlineStr"/>
-      <c r="KK3" s="1" t="inlineStr"/>
-      <c r="KL3" s="1" t="inlineStr"/>
-      <c r="KM3" s="1" t="inlineStr"/>
-      <c r="KN3" s="1" t="inlineStr"/>
-      <c r="KO3" s="1" t="inlineStr"/>
-      <c r="KP3" s="1" t="inlineStr"/>
-      <c r="KQ3" s="1" t="inlineStr"/>
-      <c r="KR3" s="1" t="inlineStr"/>
-      <c r="KS3" s="1" t="inlineStr"/>
-      <c r="KT3" s="1" t="inlineStr"/>
-      <c r="KU3" s="1" t="inlineStr"/>
-      <c r="KV3" s="1" t="inlineStr"/>
-      <c r="KW3" s="1" t="inlineStr"/>
-      <c r="KX3" s="1" t="inlineStr"/>
-      <c r="KY3" s="1" t="inlineStr"/>
-      <c r="KZ3" s="1" t="inlineStr"/>
-      <c r="LA3" s="1" t="inlineStr"/>
-      <c r="LB3" s="1" t="inlineStr"/>
-      <c r="LC3" s="1" t="inlineStr"/>
-      <c r="LD3" s="1" t="inlineStr"/>
-      <c r="LE3" s="1" t="inlineStr"/>
-      <c r="LF3" s="1" t="inlineStr"/>
-      <c r="LG3" s="1" t="inlineStr"/>
-      <c r="LH3" s="1" t="inlineStr"/>
-      <c r="LI3" s="1" t="inlineStr"/>
-      <c r="LJ3" s="1" t="inlineStr"/>
-      <c r="LK3" s="1" t="inlineStr"/>
-      <c r="LL3" s="1" t="inlineStr"/>
-      <c r="LM3" s="1" t="inlineStr"/>
-      <c r="LN3" s="1" t="inlineStr"/>
-      <c r="LO3" s="1" t="inlineStr"/>
-      <c r="LP3" s="1" t="inlineStr"/>
-      <c r="LQ3" s="1" t="inlineStr"/>
-      <c r="LR3" s="1" t="inlineStr"/>
-      <c r="LS3" s="1" t="inlineStr"/>
-      <c r="LT3" s="1" t="inlineStr"/>
-      <c r="LU3" s="1" t="inlineStr"/>
-      <c r="LV3" s="1" t="inlineStr"/>
-      <c r="LW3" s="1" t="inlineStr"/>
-      <c r="LX3" s="1" t="inlineStr"/>
-      <c r="LY3" s="1" t="inlineStr"/>
-      <c r="LZ3" s="1" t="inlineStr"/>
-      <c r="MA3" s="1" t="inlineStr"/>
-      <c r="MB3" s="1" t="inlineStr"/>
-      <c r="MC3" s="1" t="inlineStr"/>
-      <c r="MD3" s="1" t="inlineStr"/>
-      <c r="ME3" s="1" t="inlineStr"/>
-      <c r="MF3" s="1" t="inlineStr"/>
-      <c r="MG3" s="1" t="inlineStr"/>
-      <c r="MH3" s="1" t="inlineStr"/>
-      <c r="MI3" s="1" t="inlineStr"/>
-      <c r="MJ3" s="1" t="inlineStr"/>
-      <c r="MK3" s="1" t="inlineStr"/>
-      <c r="ML3" s="1" t="inlineStr"/>
-      <c r="MM3" s="1" t="inlineStr"/>
-      <c r="MN3" s="1" t="inlineStr"/>
-      <c r="MO3" s="1" t="inlineStr"/>
-      <c r="MP3" s="1" t="inlineStr"/>
-      <c r="MQ3" s="1" t="inlineStr"/>
-      <c r="MR3" s="1" t="inlineStr"/>
-      <c r="MS3" s="1" t="inlineStr"/>
-      <c r="MT3" s="1" t="inlineStr"/>
-      <c r="MU3" s="1" t="inlineStr"/>
-      <c r="MV3" s="1" t="inlineStr"/>
-      <c r="MW3" s="1" t="inlineStr"/>
-      <c r="MX3" s="1" t="inlineStr"/>
-      <c r="MY3" s="1" t="inlineStr"/>
-      <c r="MZ3" s="1" t="inlineStr"/>
-      <c r="NA3" s="1" t="inlineStr"/>
-      <c r="NB3" s="1" t="inlineStr"/>
-      <c r="NC3" s="1" t="inlineStr"/>
-      <c r="ND3" s="1" t="inlineStr"/>
-      <c r="NE3" s="1" t="inlineStr"/>
-      <c r="NF3" s="1" t="inlineStr"/>
-      <c r="NG3" s="1" t="inlineStr"/>
-      <c r="NH3" s="1" t="inlineStr"/>
-      <c r="NI3" s="1" t="inlineStr"/>
-      <c r="NJ3" s="1" t="inlineStr"/>
-      <c r="NK3" s="1" t="inlineStr"/>
-      <c r="NL3" s="1" t="inlineStr"/>
-      <c r="NM3" s="1" t="inlineStr"/>
-      <c r="NN3" s="1" t="inlineStr"/>
-      <c r="NO3" s="1" t="inlineStr"/>
-      <c r="NP3" s="1" t="inlineStr"/>
-      <c r="NQ3" s="1" t="inlineStr"/>
-      <c r="NR3" s="1" t="inlineStr"/>
-      <c r="NS3" s="1" t="inlineStr"/>
-      <c r="NT3" s="1" t="inlineStr"/>
-      <c r="NU3" s="1" t="inlineStr"/>
-      <c r="NV3" s="1" t="inlineStr"/>
-      <c r="NW3" s="1" t="inlineStr"/>
-      <c r="NX3" s="1" t="inlineStr"/>
-      <c r="NY3" s="1" t="inlineStr"/>
-      <c r="NZ3" s="1" t="inlineStr"/>
-      <c r="OA3" s="1" t="inlineStr"/>
-      <c r="OB3" s="1" t="inlineStr"/>
-      <c r="OC3" s="1" t="inlineStr"/>
-      <c r="OD3" s="1" t="inlineStr"/>
-      <c r="OE3" s="1" t="inlineStr"/>
-      <c r="OF3" s="1" t="inlineStr"/>
-      <c r="OG3" s="1" t="inlineStr"/>
-      <c r="OH3" s="1" t="inlineStr"/>
-      <c r="OI3" s="1" t="inlineStr"/>
-      <c r="OJ3" s="1" t="inlineStr"/>
-      <c r="OK3" s="1" t="inlineStr"/>
-      <c r="OL3" s="1" t="inlineStr"/>
-      <c r="OM3" s="1" t="inlineStr"/>
-      <c r="ON3" s="1" t="inlineStr"/>
-      <c r="OO3" s="1" t="inlineStr"/>
-      <c r="OP3" s="1" t="inlineStr"/>
-      <c r="OQ3" s="1" t="inlineStr"/>
-      <c r="OR3" s="1" t="inlineStr"/>
-      <c r="OS3" s="1" t="inlineStr"/>
-      <c r="OT3" s="1" t="inlineStr"/>
-      <c r="OU3" s="1" t="inlineStr"/>
-      <c r="OV3" s="1" t="inlineStr"/>
-      <c r="OW3" s="1" t="inlineStr"/>
-      <c r="OX3" s="1" t="inlineStr"/>
-      <c r="OY3" s="1" t="inlineStr"/>
-      <c r="OZ3" s="1" t="inlineStr"/>
-      <c r="PA3" s="1" t="inlineStr"/>
-      <c r="PB3" s="1" t="inlineStr"/>
-      <c r="PC3" s="1" t="inlineStr"/>
-      <c r="PD3" s="1" t="inlineStr"/>
-      <c r="PE3" s="1" t="inlineStr"/>
-      <c r="PF3" s="1" t="inlineStr"/>
-      <c r="PG3" s="1" t="inlineStr"/>
-      <c r="PH3" s="1" t="inlineStr"/>
-      <c r="PI3" s="1" t="inlineStr"/>
-      <c r="PJ3" s="1" t="inlineStr"/>
-      <c r="PK3" s="1" t="inlineStr"/>
-      <c r="PL3" s="1" t="inlineStr"/>
-      <c r="PM3" s="1" t="inlineStr"/>
-      <c r="PN3" s="1" t="inlineStr"/>
-      <c r="PO3" s="1" t="inlineStr"/>
-      <c r="PP3" s="1" t="inlineStr"/>
-      <c r="PQ3" s="1" t="inlineStr"/>
-      <c r="PR3" s="1" t="inlineStr"/>
-      <c r="PS3" s="1" t="inlineStr"/>
-      <c r="PT3" s="1" t="inlineStr"/>
-      <c r="PU3" s="1" t="inlineStr"/>
-      <c r="PV3" s="1" t="inlineStr"/>
-      <c r="PW3" s="1" t="inlineStr"/>
-      <c r="PX3" s="1" t="inlineStr"/>
-      <c r="PY3" s="1" t="inlineStr"/>
-      <c r="PZ3" s="1" t="inlineStr"/>
-      <c r="QA3" s="1" t="inlineStr"/>
-      <c r="QB3" s="1" t="inlineStr"/>
-      <c r="QC3" s="1" t="inlineStr"/>
-      <c r="QD3" s="1" t="inlineStr"/>
-      <c r="QE3" s="1" t="inlineStr"/>
-      <c r="QF3" s="1" t="inlineStr"/>
-      <c r="QG3" s="1" t="inlineStr"/>
-      <c r="QH3" s="1" t="inlineStr"/>
-      <c r="QI3" s="1" t="inlineStr"/>
-      <c r="QJ3" s="1" t="inlineStr"/>
-      <c r="QK3" s="1" t="inlineStr"/>
-      <c r="QL3" s="1" t="inlineStr"/>
-      <c r="QM3" s="1" t="inlineStr"/>
-      <c r="QN3" s="1" t="inlineStr"/>
-      <c r="QO3" s="1" t="inlineStr"/>
-      <c r="QP3" s="1" t="inlineStr"/>
-      <c r="QQ3" s="1" t="inlineStr"/>
-      <c r="QR3" s="1" t="inlineStr"/>
-      <c r="QS3" s="1" t="inlineStr"/>
-      <c r="QT3" s="1" t="inlineStr"/>
-      <c r="QU3" s="1" t="inlineStr"/>
-      <c r="QV3" s="1" t="inlineStr"/>
-      <c r="QW3" s="1" t="inlineStr"/>
+      <c r="B3" s="2" t="inlineStr"/>
+      <c r="C3" s="2" t="inlineStr"/>
+      <c r="D3" s="2" t="inlineStr"/>
+      <c r="E3" s="2" t="inlineStr"/>
+      <c r="F3" s="2" t="inlineStr"/>
+      <c r="G3" s="2" t="inlineStr"/>
+      <c r="H3" s="2" t="inlineStr"/>
+      <c r="I3" s="2" t="inlineStr"/>
+      <c r="J3" s="2" t="inlineStr"/>
+      <c r="K3" s="2" t="inlineStr"/>
+      <c r="L3" s="2" t="inlineStr"/>
+      <c r="M3" s="2" t="inlineStr"/>
+      <c r="N3" s="2" t="inlineStr"/>
+      <c r="O3" s="2" t="inlineStr"/>
+      <c r="P3" s="2" t="inlineStr"/>
+      <c r="Q3" s="2" t="inlineStr"/>
+      <c r="R3" s="2" t="inlineStr"/>
+      <c r="S3" s="2" t="inlineStr"/>
+      <c r="T3" s="2" t="inlineStr"/>
+      <c r="U3" s="2" t="inlineStr"/>
+      <c r="V3" s="2" t="inlineStr"/>
+      <c r="W3" s="2" t="inlineStr"/>
+      <c r="X3" s="2" t="inlineStr"/>
+      <c r="Y3" s="2" t="inlineStr"/>
+      <c r="Z3" s="2" t="inlineStr"/>
+      <c r="AA3" s="2" t="inlineStr"/>
+      <c r="AB3" s="2" t="inlineStr"/>
+      <c r="AC3" s="2" t="inlineStr"/>
+      <c r="AD3" s="2" t="inlineStr"/>
+      <c r="AE3" s="2" t="inlineStr"/>
+      <c r="AF3" s="2" t="inlineStr"/>
+      <c r="AG3" s="2" t="inlineStr"/>
+      <c r="AH3" s="2" t="inlineStr"/>
+      <c r="AI3" s="2" t="inlineStr"/>
+      <c r="AJ3" s="2" t="inlineStr"/>
+      <c r="AK3" s="2" t="inlineStr"/>
+      <c r="AL3" s="2" t="inlineStr"/>
+      <c r="AM3" s="2" t="inlineStr"/>
+      <c r="AN3" s="2" t="inlineStr"/>
+      <c r="AO3" s="2" t="inlineStr"/>
+      <c r="AP3" s="2" t="inlineStr"/>
+      <c r="AQ3" s="2" t="inlineStr"/>
+      <c r="AR3" s="2" t="inlineStr"/>
+      <c r="AS3" s="2" t="inlineStr"/>
+      <c r="AT3" s="2" t="inlineStr"/>
+      <c r="AU3" s="2" t="inlineStr"/>
+      <c r="AV3" s="2" t="inlineStr"/>
+      <c r="AW3" s="2" t="inlineStr"/>
+      <c r="AX3" s="2" t="inlineStr"/>
+      <c r="AY3" s="2" t="inlineStr"/>
+      <c r="AZ3" s="2" t="inlineStr"/>
+      <c r="BA3" s="2" t="inlineStr"/>
+      <c r="BB3" s="2" t="inlineStr"/>
+      <c r="BC3" s="2" t="inlineStr"/>
+      <c r="BD3" s="2" t="inlineStr"/>
+      <c r="BE3" s="2" t="inlineStr"/>
+      <c r="BF3" s="2" t="inlineStr"/>
+      <c r="BG3" s="2" t="inlineStr"/>
+      <c r="BH3" s="2" t="inlineStr"/>
+      <c r="BI3" s="2" t="inlineStr"/>
+      <c r="BJ3" s="2" t="inlineStr"/>
+      <c r="BK3" s="2" t="inlineStr"/>
+      <c r="BL3" s="2" t="inlineStr"/>
+      <c r="BM3" s="2" t="inlineStr"/>
+      <c r="BN3" s="2" t="inlineStr"/>
+      <c r="BO3" s="2" t="inlineStr"/>
+      <c r="BP3" s="2" t="inlineStr"/>
+      <c r="BQ3" s="2" t="inlineStr"/>
+      <c r="BR3" s="2" t="inlineStr"/>
+      <c r="BS3" s="2" t="inlineStr"/>
+      <c r="BT3" s="2" t="inlineStr"/>
+      <c r="BU3" s="2" t="inlineStr"/>
+      <c r="BV3" s="2" t="inlineStr"/>
+      <c r="BW3" s="2" t="inlineStr"/>
+      <c r="BX3" s="2" t="inlineStr"/>
+      <c r="BY3" s="2" t="inlineStr"/>
+      <c r="BZ3" s="2" t="inlineStr"/>
+      <c r="CA3" s="2" t="inlineStr"/>
+      <c r="CB3" s="2" t="inlineStr"/>
+      <c r="CC3" s="2" t="inlineStr"/>
+      <c r="CD3" s="2" t="inlineStr"/>
+      <c r="CE3" s="2" t="inlineStr"/>
+      <c r="CF3" s="2" t="inlineStr"/>
+      <c r="CG3" s="2" t="inlineStr"/>
+      <c r="CH3" s="2" t="inlineStr"/>
+      <c r="CI3" s="2" t="inlineStr"/>
+      <c r="CJ3" s="2" t="inlineStr"/>
+      <c r="CK3" s="2" t="inlineStr"/>
+      <c r="CL3" s="2" t="inlineStr"/>
+      <c r="CM3" s="2" t="inlineStr"/>
+      <c r="CN3" s="2" t="inlineStr"/>
+      <c r="CO3" s="2" t="inlineStr"/>
+      <c r="CP3" s="2" t="inlineStr"/>
+      <c r="CQ3" s="2" t="inlineStr"/>
+      <c r="CR3" s="2" t="inlineStr"/>
+      <c r="CS3" s="2" t="inlineStr"/>
+      <c r="CT3" s="2" t="inlineStr"/>
+      <c r="CU3" s="2" t="inlineStr"/>
+      <c r="CV3" s="2" t="inlineStr"/>
+      <c r="CW3" s="2" t="inlineStr"/>
+      <c r="CX3" s="2" t="inlineStr"/>
+      <c r="CY3" s="2" t="inlineStr"/>
+      <c r="CZ3" s="2" t="inlineStr"/>
+      <c r="DA3" s="2" t="inlineStr"/>
+      <c r="DB3" s="2" t="inlineStr"/>
+      <c r="DC3" s="2" t="inlineStr"/>
+      <c r="DD3" s="2" t="inlineStr"/>
+      <c r="DE3" s="2" t="inlineStr"/>
+      <c r="DF3" s="2" t="inlineStr"/>
+      <c r="DG3" s="2" t="inlineStr"/>
+      <c r="DH3" s="2" t="inlineStr"/>
+      <c r="DI3" s="2" t="inlineStr"/>
+      <c r="DJ3" s="2" t="inlineStr"/>
+      <c r="DK3" s="2" t="inlineStr"/>
+      <c r="DL3" s="2" t="inlineStr"/>
+      <c r="DM3" s="2" t="inlineStr"/>
+      <c r="DN3" s="2" t="inlineStr"/>
+      <c r="DO3" s="2" t="inlineStr"/>
+      <c r="DP3" s="2" t="inlineStr"/>
+      <c r="DQ3" s="2" t="inlineStr"/>
+      <c r="DR3" s="2" t="inlineStr"/>
+      <c r="DS3" s="2" t="inlineStr"/>
+      <c r="DT3" s="2" t="inlineStr"/>
+      <c r="DU3" s="2" t="inlineStr"/>
+      <c r="DV3" s="2" t="inlineStr"/>
+      <c r="DW3" s="2" t="inlineStr"/>
+      <c r="DX3" s="2" t="inlineStr"/>
+      <c r="DY3" s="2" t="inlineStr"/>
+      <c r="DZ3" s="2" t="inlineStr"/>
+      <c r="EA3" s="2" t="inlineStr"/>
+      <c r="EB3" s="2" t="inlineStr"/>
+      <c r="EC3" s="2" t="inlineStr"/>
+      <c r="ED3" s="2" t="inlineStr"/>
+      <c r="EE3" s="2" t="inlineStr"/>
+      <c r="EF3" s="2" t="inlineStr"/>
+      <c r="EG3" s="2" t="inlineStr"/>
+      <c r="EH3" s="2" t="inlineStr"/>
+      <c r="EI3" s="2" t="inlineStr"/>
+      <c r="EJ3" s="2" t="inlineStr"/>
+      <c r="EK3" s="2" t="inlineStr"/>
+      <c r="EL3" s="2" t="inlineStr"/>
+      <c r="EM3" s="2" t="inlineStr"/>
+      <c r="EN3" s="2" t="inlineStr"/>
+      <c r="EO3" s="2" t="inlineStr"/>
+      <c r="EP3" s="2" t="inlineStr"/>
+      <c r="EQ3" s="2" t="inlineStr"/>
+      <c r="ER3" s="2" t="inlineStr"/>
+      <c r="ES3" s="2" t="inlineStr"/>
+      <c r="ET3" s="2" t="inlineStr"/>
+      <c r="EU3" s="2" t="inlineStr"/>
+      <c r="EV3" s="2" t="inlineStr"/>
+      <c r="EW3" s="2" t="inlineStr"/>
+      <c r="EX3" s="2" t="inlineStr"/>
+      <c r="EY3" s="2" t="inlineStr"/>
+      <c r="EZ3" s="2" t="inlineStr"/>
+      <c r="FA3" s="2" t="inlineStr"/>
+      <c r="FB3" s="2" t="inlineStr"/>
+      <c r="FC3" s="2" t="inlineStr"/>
+      <c r="FD3" s="2" t="inlineStr"/>
+      <c r="FE3" s="2" t="inlineStr"/>
+      <c r="FF3" s="2" t="inlineStr"/>
+      <c r="FG3" s="2" t="inlineStr"/>
+      <c r="FH3" s="2" t="inlineStr"/>
+      <c r="FI3" s="2" t="inlineStr"/>
+      <c r="FJ3" s="2" t="inlineStr"/>
+      <c r="FK3" s="2" t="inlineStr"/>
+      <c r="FL3" s="2" t="inlineStr"/>
+      <c r="FM3" s="2" t="inlineStr"/>
+      <c r="FN3" s="2" t="inlineStr"/>
+      <c r="FO3" s="2" t="inlineStr"/>
+      <c r="FP3" s="2" t="inlineStr"/>
+      <c r="FQ3" s="2" t="inlineStr"/>
+      <c r="FR3" s="2" t="inlineStr"/>
+      <c r="FS3" s="2" t="inlineStr"/>
+      <c r="FT3" s="2" t="inlineStr"/>
+      <c r="FU3" s="2" t="inlineStr"/>
+      <c r="FV3" s="2" t="inlineStr"/>
+      <c r="FW3" s="2" t="inlineStr"/>
+      <c r="FX3" s="2" t="inlineStr"/>
+      <c r="FY3" s="2" t="inlineStr"/>
+      <c r="FZ3" s="2" t="inlineStr"/>
+      <c r="GA3" s="2" t="inlineStr"/>
+      <c r="GB3" s="2" t="inlineStr"/>
+      <c r="GC3" s="2" t="inlineStr"/>
+      <c r="GD3" s="2" t="inlineStr"/>
+      <c r="GE3" s="2" t="inlineStr"/>
+      <c r="GF3" s="2" t="inlineStr"/>
+      <c r="GG3" s="2" t="inlineStr"/>
+      <c r="GH3" s="2" t="inlineStr"/>
+      <c r="GI3" s="2" t="inlineStr"/>
+      <c r="GJ3" s="2" t="inlineStr"/>
+      <c r="GK3" s="2" t="inlineStr"/>
+      <c r="GL3" s="2" t="inlineStr"/>
+      <c r="GM3" s="2" t="inlineStr"/>
+      <c r="GN3" s="2" t="inlineStr"/>
+      <c r="GO3" s="2" t="inlineStr"/>
+      <c r="GP3" s="2" t="inlineStr"/>
+      <c r="GQ3" s="2" t="inlineStr"/>
+      <c r="GR3" s="2" t="inlineStr"/>
+      <c r="GS3" s="2" t="inlineStr"/>
+      <c r="GT3" s="2" t="inlineStr"/>
+      <c r="GU3" s="2" t="inlineStr"/>
+      <c r="GV3" s="2" t="inlineStr"/>
+      <c r="GW3" s="2" t="inlineStr"/>
+      <c r="GX3" s="2" t="inlineStr"/>
+      <c r="GY3" s="2" t="inlineStr"/>
+      <c r="GZ3" s="2" t="inlineStr"/>
+      <c r="HA3" s="2" t="inlineStr"/>
+      <c r="HB3" s="2" t="inlineStr"/>
+      <c r="HC3" s="2" t="inlineStr"/>
+      <c r="HD3" s="2" t="inlineStr"/>
+      <c r="HE3" s="2" t="inlineStr"/>
+      <c r="HF3" s="2" t="inlineStr"/>
+      <c r="HG3" s="2" t="inlineStr"/>
+      <c r="HH3" s="2" t="inlineStr"/>
+      <c r="HI3" s="2" t="inlineStr"/>
+      <c r="HJ3" s="2" t="inlineStr"/>
+      <c r="HK3" s="2" t="inlineStr"/>
+      <c r="HL3" s="2" t="inlineStr"/>
+      <c r="HM3" s="2" t="inlineStr"/>
+      <c r="HN3" s="2" t="inlineStr"/>
+      <c r="HO3" s="2" t="inlineStr"/>
+      <c r="HP3" s="2" t="inlineStr"/>
+      <c r="HQ3" s="2" t="inlineStr"/>
+      <c r="HR3" s="2" t="inlineStr"/>
+      <c r="HS3" s="2" t="inlineStr"/>
+      <c r="HT3" s="2" t="inlineStr"/>
+      <c r="HU3" s="2" t="inlineStr"/>
+      <c r="HV3" s="2" t="inlineStr"/>
+      <c r="HW3" s="2" t="inlineStr"/>
+      <c r="HX3" s="2" t="inlineStr"/>
+      <c r="HY3" s="2" t="inlineStr"/>
+      <c r="HZ3" s="2" t="inlineStr"/>
+      <c r="IA3" s="2" t="inlineStr"/>
+      <c r="IB3" s="2" t="inlineStr"/>
+      <c r="IC3" s="2" t="inlineStr"/>
+      <c r="ID3" s="2" t="inlineStr"/>
+      <c r="IE3" s="2" t="inlineStr"/>
+      <c r="IF3" s="2" t="inlineStr"/>
+      <c r="IG3" s="2" t="inlineStr"/>
+      <c r="IH3" s="2" t="inlineStr"/>
+      <c r="II3" s="2" t="inlineStr"/>
+      <c r="IJ3" s="2" t="inlineStr"/>
+      <c r="IK3" s="2" t="inlineStr"/>
+      <c r="IL3" s="2" t="inlineStr"/>
+      <c r="IM3" s="2" t="inlineStr"/>
+      <c r="IN3" s="2" t="inlineStr"/>
+      <c r="IO3" s="2" t="inlineStr"/>
+      <c r="IP3" s="2" t="inlineStr"/>
+      <c r="IQ3" s="2" t="inlineStr"/>
+      <c r="IR3" s="2" t="inlineStr"/>
+      <c r="IS3" s="2" t="inlineStr"/>
+      <c r="IT3" s="2" t="inlineStr"/>
+      <c r="IU3" s="2" t="inlineStr"/>
+      <c r="IV3" s="2" t="inlineStr"/>
+      <c r="IW3" s="2" t="inlineStr"/>
+      <c r="IX3" s="2" t="inlineStr"/>
+      <c r="IY3" s="2" t="inlineStr"/>
+      <c r="IZ3" s="2" t="inlineStr"/>
+      <c r="JA3" s="2" t="inlineStr"/>
+      <c r="JB3" s="2" t="inlineStr"/>
+      <c r="JC3" s="2" t="inlineStr"/>
+      <c r="JD3" s="2" t="inlineStr"/>
+      <c r="JE3" s="2" t="inlineStr"/>
+      <c r="JF3" s="2" t="inlineStr"/>
+      <c r="JG3" s="2" t="inlineStr"/>
+      <c r="JH3" s="2" t="inlineStr"/>
+      <c r="JI3" s="2" t="inlineStr"/>
+      <c r="JJ3" s="2" t="inlineStr"/>
+      <c r="JK3" s="2" t="inlineStr"/>
+      <c r="JL3" s="2" t="inlineStr"/>
+      <c r="JM3" s="2" t="inlineStr"/>
+      <c r="JN3" s="2" t="inlineStr"/>
+      <c r="JO3" s="2" t="inlineStr"/>
+      <c r="JP3" s="2" t="inlineStr"/>
+      <c r="JQ3" s="2" t="inlineStr"/>
+      <c r="JR3" s="2" t="inlineStr"/>
+      <c r="JS3" s="2" t="inlineStr"/>
+      <c r="JT3" s="2" t="inlineStr"/>
+      <c r="JU3" s="2" t="inlineStr"/>
+      <c r="JV3" s="2" t="inlineStr"/>
+      <c r="JW3" s="2" t="inlineStr"/>
+      <c r="JX3" s="2" t="inlineStr"/>
+      <c r="JY3" s="2" t="inlineStr"/>
+      <c r="JZ3" s="2" t="inlineStr"/>
+      <c r="KA3" s="2" t="inlineStr"/>
+      <c r="KB3" s="2" t="inlineStr"/>
+      <c r="KC3" s="2" t="inlineStr"/>
+      <c r="KD3" s="2" t="inlineStr"/>
+      <c r="KE3" s="2" t="inlineStr"/>
+      <c r="KF3" s="2" t="inlineStr"/>
+      <c r="KG3" s="2" t="inlineStr"/>
+      <c r="KH3" s="2" t="inlineStr"/>
+      <c r="KI3" s="2" t="inlineStr"/>
+      <c r="KJ3" s="2" t="inlineStr"/>
+      <c r="KK3" s="2" t="inlineStr"/>
+      <c r="KL3" s="2" t="inlineStr"/>
+      <c r="KM3" s="2" t="inlineStr"/>
+      <c r="KN3" s="2" t="inlineStr"/>
+      <c r="KO3" s="2" t="inlineStr"/>
+      <c r="KP3" s="2" t="inlineStr"/>
+      <c r="KQ3" s="2" t="inlineStr"/>
+      <c r="KR3" s="2" t="inlineStr"/>
+      <c r="KS3" s="2" t="inlineStr"/>
+      <c r="KT3" s="2" t="inlineStr"/>
+      <c r="KU3" s="2" t="inlineStr"/>
+      <c r="KV3" s="2" t="inlineStr"/>
+      <c r="KW3" s="2" t="inlineStr"/>
+      <c r="KX3" s="2" t="inlineStr"/>
+      <c r="KY3" s="2" t="inlineStr"/>
+      <c r="KZ3" s="2" t="inlineStr"/>
+      <c r="LA3" s="2" t="inlineStr"/>
+      <c r="LB3" s="2" t="inlineStr"/>
+      <c r="LC3" s="2" t="inlineStr"/>
+      <c r="LD3" s="2" t="inlineStr"/>
+      <c r="LE3" s="2" t="inlineStr"/>
+      <c r="LF3" s="2" t="inlineStr"/>
+      <c r="LG3" s="2" t="inlineStr"/>
+      <c r="LH3" s="2" t="inlineStr"/>
+      <c r="LI3" s="2" t="inlineStr"/>
+      <c r="LJ3" s="2" t="inlineStr"/>
+      <c r="LK3" s="2" t="inlineStr"/>
+      <c r="LL3" s="2" t="inlineStr"/>
+      <c r="LM3" s="2" t="inlineStr"/>
+      <c r="LN3" s="2" t="inlineStr"/>
+      <c r="LO3" s="2" t="inlineStr"/>
+      <c r="LP3" s="2" t="inlineStr"/>
+      <c r="LQ3" s="2" t="inlineStr"/>
+      <c r="LR3" s="2" t="inlineStr"/>
+      <c r="LS3" s="2" t="inlineStr"/>
+      <c r="LT3" s="2" t="inlineStr"/>
+      <c r="LU3" s="2" t="inlineStr"/>
+      <c r="LV3" s="2" t="inlineStr"/>
+      <c r="LW3" s="2" t="inlineStr"/>
+      <c r="LX3" s="2" t="inlineStr"/>
+      <c r="LY3" s="2" t="inlineStr"/>
+      <c r="LZ3" s="2" t="inlineStr"/>
+      <c r="MA3" s="2" t="inlineStr"/>
+      <c r="MB3" s="2" t="inlineStr"/>
+      <c r="MC3" s="2" t="inlineStr"/>
+      <c r="MD3" s="2" t="inlineStr"/>
+      <c r="ME3" s="2" t="inlineStr"/>
+      <c r="MF3" s="2" t="inlineStr"/>
+      <c r="MG3" s="2" t="inlineStr"/>
+      <c r="MH3" s="2" t="inlineStr"/>
+      <c r="MI3" s="2" t="inlineStr"/>
+      <c r="MJ3" s="2" t="inlineStr"/>
+      <c r="MK3" s="2" t="inlineStr"/>
+      <c r="ML3" s="2" t="inlineStr"/>
+      <c r="MM3" s="2" t="inlineStr"/>
+      <c r="MN3" s="2" t="inlineStr"/>
+      <c r="MO3" s="2" t="inlineStr"/>
+      <c r="MP3" s="2" t="inlineStr"/>
+      <c r="MQ3" s="2" t="inlineStr"/>
+      <c r="MR3" s="2" t="inlineStr"/>
+      <c r="MS3" s="2" t="inlineStr"/>
+      <c r="MT3" s="2" t="inlineStr"/>
+      <c r="MU3" s="2" t="inlineStr"/>
+      <c r="MV3" s="2" t="inlineStr"/>
+      <c r="MW3" s="2" t="inlineStr"/>
+      <c r="MX3" s="2" t="inlineStr"/>
+      <c r="MY3" s="2" t="inlineStr"/>
+      <c r="MZ3" s="2" t="inlineStr"/>
+      <c r="NA3" s="2" t="inlineStr"/>
+      <c r="NB3" s="2" t="inlineStr"/>
+      <c r="NC3" s="2" t="inlineStr"/>
+      <c r="ND3" s="2" t="inlineStr"/>
+      <c r="NE3" s="2" t="inlineStr"/>
+      <c r="NF3" s="2" t="inlineStr"/>
+      <c r="NG3" s="2" t="inlineStr"/>
+      <c r="NH3" s="2" t="inlineStr"/>
+      <c r="NI3" s="2" t="inlineStr"/>
+      <c r="NJ3" s="2" t="inlineStr"/>
+      <c r="NK3" s="2" t="inlineStr"/>
+      <c r="NL3" s="2" t="inlineStr"/>
+      <c r="NM3" s="2" t="inlineStr"/>
+      <c r="NN3" s="2" t="inlineStr"/>
+      <c r="NO3" s="2" t="inlineStr"/>
+      <c r="NP3" s="2" t="inlineStr"/>
+      <c r="NQ3" s="2" t="inlineStr"/>
+      <c r="NR3" s="2" t="inlineStr"/>
+      <c r="NS3" s="2" t="inlineStr"/>
+      <c r="NT3" s="2" t="inlineStr"/>
+      <c r="NU3" s="2" t="inlineStr"/>
+      <c r="NV3" s="2" t="inlineStr"/>
+      <c r="NW3" s="2" t="inlineStr"/>
+      <c r="NX3" s="2" t="inlineStr"/>
+      <c r="NY3" s="2" t="inlineStr"/>
+      <c r="NZ3" s="2" t="inlineStr"/>
+      <c r="OA3" s="2" t="inlineStr"/>
+      <c r="OB3" s="2" t="inlineStr"/>
+      <c r="OC3" s="2" t="inlineStr"/>
+      <c r="OD3" s="2" t="inlineStr"/>
+      <c r="OE3" s="2" t="inlineStr"/>
+      <c r="OF3" s="2" t="inlineStr"/>
+      <c r="OG3" s="2" t="inlineStr"/>
+      <c r="OH3" s="2" t="inlineStr"/>
+      <c r="OI3" s="2" t="inlineStr"/>
+      <c r="OJ3" s="2" t="inlineStr"/>
+      <c r="OK3" s="2" t="inlineStr"/>
+      <c r="OL3" s="2" t="inlineStr"/>
+      <c r="OM3" s="2" t="inlineStr"/>
+      <c r="ON3" s="2" t="inlineStr"/>
+      <c r="OO3" s="2" t="inlineStr"/>
+      <c r="OP3" s="2" t="inlineStr"/>
+      <c r="OQ3" s="2" t="inlineStr"/>
+      <c r="OR3" s="2" t="inlineStr"/>
+      <c r="OS3" s="2" t="inlineStr"/>
+      <c r="OT3" s="2" t="inlineStr"/>
+      <c r="OU3" s="2" t="inlineStr"/>
+      <c r="OV3" s="2" t="inlineStr"/>
+      <c r="OW3" s="2" t="inlineStr"/>
+      <c r="OX3" s="2" t="inlineStr"/>
+      <c r="OY3" s="2" t="inlineStr"/>
+      <c r="OZ3" s="2" t="inlineStr"/>
+      <c r="PA3" s="2" t="inlineStr"/>
+      <c r="PB3" s="2" t="inlineStr"/>
+      <c r="PC3" s="2" t="inlineStr"/>
+      <c r="PD3" s="2" t="inlineStr"/>
+      <c r="PE3" s="2" t="inlineStr"/>
+      <c r="PF3" s="2" t="inlineStr"/>
+      <c r="PG3" s="2" t="inlineStr"/>
+      <c r="PH3" s="2" t="inlineStr"/>
+      <c r="PI3" s="2" t="inlineStr"/>
+      <c r="PJ3" s="2" t="inlineStr"/>
+      <c r="PK3" s="2" t="inlineStr"/>
+      <c r="PL3" s="2" t="inlineStr"/>
+      <c r="PM3" s="2" t="inlineStr"/>
+      <c r="PN3" s="2" t="inlineStr"/>
+      <c r="PO3" s="2" t="inlineStr"/>
+      <c r="PP3" s="2" t="inlineStr"/>
+      <c r="PQ3" s="2" t="inlineStr"/>
+      <c r="PR3" s="2" t="inlineStr"/>
+      <c r="PS3" s="2" t="inlineStr"/>
+      <c r="PT3" s="2" t="inlineStr"/>
+      <c r="PU3" s="2" t="inlineStr"/>
+      <c r="PV3" s="2" t="inlineStr"/>
+      <c r="PW3" s="2" t="inlineStr"/>
+      <c r="PX3" s="2" t="inlineStr"/>
+      <c r="PY3" s="2" t="inlineStr"/>
+      <c r="PZ3" s="2" t="inlineStr"/>
+      <c r="QA3" s="2" t="inlineStr"/>
+      <c r="QB3" s="2" t="inlineStr"/>
+      <c r="QC3" s="2" t="inlineStr"/>
+      <c r="QD3" s="2" t="inlineStr"/>
+      <c r="QE3" s="2" t="inlineStr"/>
+      <c r="QF3" s="2" t="inlineStr"/>
+      <c r="QG3" s="2" t="inlineStr"/>
+      <c r="QH3" s="2" t="inlineStr"/>
+      <c r="QI3" s="2" t="inlineStr"/>
+      <c r="QJ3" s="2" t="inlineStr"/>
+      <c r="QK3" s="2" t="inlineStr"/>
+      <c r="QL3" s="2" t="inlineStr"/>
+      <c r="QM3" s="2" t="inlineStr"/>
+      <c r="QN3" s="2" t="inlineStr"/>
+      <c r="QO3" s="2" t="inlineStr"/>
+      <c r="QP3" s="2" t="inlineStr"/>
+      <c r="QQ3" s="2" t="inlineStr"/>
+      <c r="QR3" s="2" t="inlineStr"/>
+      <c r="QS3" s="2" t="inlineStr"/>
+      <c r="QT3" s="2" t="inlineStr"/>
+      <c r="QU3" s="2" t="inlineStr"/>
+      <c r="QV3" s="2" t="inlineStr"/>
+      <c r="QW3" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>